<commit_message>
feat(#25): T5 Anslag tab in the sheet template
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Grupper" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tränare" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Säsonger" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Anslag" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11282,4 +11283,1862 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D300"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Meddelande</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Meddelande (EN)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Visa från</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Visa till</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Exempel: Kvällens träning är inställd på grund av sjukdom.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Example: Tonight's session is cancelled because the coach is ill.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="2" t="n"/>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="2" t="n"/>
+      <c r="C98" s="2" t="n"/>
+      <c r="D98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="2" t="n"/>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n"/>
+      <c r="B100" s="2" t="n"/>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n"/>
+      <c r="B101" s="2" t="n"/>
+      <c r="C101" s="2" t="n"/>
+      <c r="D101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n"/>
+      <c r="B102" s="2" t="n"/>
+      <c r="C102" s="2" t="n"/>
+      <c r="D102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n"/>
+      <c r="B103" s="2" t="n"/>
+      <c r="C103" s="2" t="n"/>
+      <c r="D103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n"/>
+      <c r="B104" s="2" t="n"/>
+      <c r="C104" s="2" t="n"/>
+      <c r="D104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n"/>
+      <c r="B105" s="2" t="n"/>
+      <c r="C105" s="2" t="n"/>
+      <c r="D105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="2" t="n"/>
+      <c r="C106" s="2" t="n"/>
+      <c r="D106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n"/>
+      <c r="B107" s="2" t="n"/>
+      <c r="C107" s="2" t="n"/>
+      <c r="D107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="2" t="n"/>
+      <c r="C108" s="2" t="n"/>
+      <c r="D108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n"/>
+      <c r="B109" s="2" t="n"/>
+      <c r="C109" s="2" t="n"/>
+      <c r="D109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n"/>
+      <c r="B110" s="2" t="n"/>
+      <c r="C110" s="2" t="n"/>
+      <c r="D110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n"/>
+      <c r="B111" s="2" t="n"/>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n"/>
+      <c r="B112" s="2" t="n"/>
+      <c r="C112" s="2" t="n"/>
+      <c r="D112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n"/>
+      <c r="B113" s="2" t="n"/>
+      <c r="C113" s="2" t="n"/>
+      <c r="D113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n"/>
+      <c r="B114" s="2" t="n"/>
+      <c r="C114" s="2" t="n"/>
+      <c r="D114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n"/>
+      <c r="B115" s="2" t="n"/>
+      <c r="C115" s="2" t="n"/>
+      <c r="D115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n"/>
+      <c r="B116" s="2" t="n"/>
+      <c r="C116" s="2" t="n"/>
+      <c r="D116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n"/>
+      <c r="B117" s="2" t="n"/>
+      <c r="C117" s="2" t="n"/>
+      <c r="D117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n"/>
+      <c r="B118" s="2" t="n"/>
+      <c r="C118" s="2" t="n"/>
+      <c r="D118" s="2" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n"/>
+      <c r="B119" s="2" t="n"/>
+      <c r="C119" s="2" t="n"/>
+      <c r="D119" s="2" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n"/>
+      <c r="B120" s="2" t="n"/>
+      <c r="C120" s="2" t="n"/>
+      <c r="D120" s="2" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n"/>
+      <c r="B121" s="2" t="n"/>
+      <c r="C121" s="2" t="n"/>
+      <c r="D121" s="2" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n"/>
+      <c r="B122" s="2" t="n"/>
+      <c r="C122" s="2" t="n"/>
+      <c r="D122" s="2" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n"/>
+      <c r="B123" s="2" t="n"/>
+      <c r="C123" s="2" t="n"/>
+      <c r="D123" s="2" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n"/>
+      <c r="B124" s="2" t="n"/>
+      <c r="C124" s="2" t="n"/>
+      <c r="D124" s="2" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n"/>
+      <c r="B125" s="2" t="n"/>
+      <c r="C125" s="2" t="n"/>
+      <c r="D125" s="2" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n"/>
+      <c r="B126" s="2" t="n"/>
+      <c r="C126" s="2" t="n"/>
+      <c r="D126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n"/>
+      <c r="B127" s="2" t="n"/>
+      <c r="C127" s="2" t="n"/>
+      <c r="D127" s="2" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n"/>
+      <c r="B128" s="2" t="n"/>
+      <c r="C128" s="2" t="n"/>
+      <c r="D128" s="2" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n"/>
+      <c r="B129" s="2" t="n"/>
+      <c r="C129" s="2" t="n"/>
+      <c r="D129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n"/>
+      <c r="B130" s="2" t="n"/>
+      <c r="C130" s="2" t="n"/>
+      <c r="D130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n"/>
+      <c r="B131" s="2" t="n"/>
+      <c r="C131" s="2" t="n"/>
+      <c r="D131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n"/>
+      <c r="B132" s="2" t="n"/>
+      <c r="C132" s="2" t="n"/>
+      <c r="D132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n"/>
+      <c r="B133" s="2" t="n"/>
+      <c r="C133" s="2" t="n"/>
+      <c r="D133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n"/>
+      <c r="B134" s="2" t="n"/>
+      <c r="C134" s="2" t="n"/>
+      <c r="D134" s="2" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n"/>
+      <c r="B135" s="2" t="n"/>
+      <c r="C135" s="2" t="n"/>
+      <c r="D135" s="2" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n"/>
+      <c r="B136" s="2" t="n"/>
+      <c r="C136" s="2" t="n"/>
+      <c r="D136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n"/>
+      <c r="B137" s="2" t="n"/>
+      <c r="C137" s="2" t="n"/>
+      <c r="D137" s="2" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n"/>
+      <c r="B138" s="2" t="n"/>
+      <c r="C138" s="2" t="n"/>
+      <c r="D138" s="2" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n"/>
+      <c r="B139" s="2" t="n"/>
+      <c r="C139" s="2" t="n"/>
+      <c r="D139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n"/>
+      <c r="B140" s="2" t="n"/>
+      <c r="C140" s="2" t="n"/>
+      <c r="D140" s="2" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n"/>
+      <c r="B141" s="2" t="n"/>
+      <c r="C141" s="2" t="n"/>
+      <c r="D141" s="2" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n"/>
+      <c r="B142" s="2" t="n"/>
+      <c r="C142" s="2" t="n"/>
+      <c r="D142" s="2" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n"/>
+      <c r="B143" s="2" t="n"/>
+      <c r="C143" s="2" t="n"/>
+      <c r="D143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n"/>
+      <c r="B144" s="2" t="n"/>
+      <c r="C144" s="2" t="n"/>
+      <c r="D144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n"/>
+      <c r="B145" s="2" t="n"/>
+      <c r="C145" s="2" t="n"/>
+      <c r="D145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n"/>
+      <c r="B146" s="2" t="n"/>
+      <c r="C146" s="2" t="n"/>
+      <c r="D146" s="2" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n"/>
+      <c r="B147" s="2" t="n"/>
+      <c r="C147" s="2" t="n"/>
+      <c r="D147" s="2" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n"/>
+      <c r="B148" s="2" t="n"/>
+      <c r="C148" s="2" t="n"/>
+      <c r="D148" s="2" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n"/>
+      <c r="B149" s="2" t="n"/>
+      <c r="C149" s="2" t="n"/>
+      <c r="D149" s="2" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n"/>
+      <c r="B150" s="2" t="n"/>
+      <c r="C150" s="2" t="n"/>
+      <c r="D150" s="2" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n"/>
+      <c r="B151" s="2" t="n"/>
+      <c r="C151" s="2" t="n"/>
+      <c r="D151" s="2" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n"/>
+      <c r="B152" s="2" t="n"/>
+      <c r="C152" s="2" t="n"/>
+      <c r="D152" s="2" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n"/>
+      <c r="B153" s="2" t="n"/>
+      <c r="C153" s="2" t="n"/>
+      <c r="D153" s="2" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n"/>
+      <c r="B154" s="2" t="n"/>
+      <c r="C154" s="2" t="n"/>
+      <c r="D154" s="2" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n"/>
+      <c r="B155" s="2" t="n"/>
+      <c r="C155" s="2" t="n"/>
+      <c r="D155" s="2" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n"/>
+      <c r="B156" s="2" t="n"/>
+      <c r="C156" s="2" t="n"/>
+      <c r="D156" s="2" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n"/>
+      <c r="B157" s="2" t="n"/>
+      <c r="C157" s="2" t="n"/>
+      <c r="D157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n"/>
+      <c r="B158" s="2" t="n"/>
+      <c r="C158" s="2" t="n"/>
+      <c r="D158" s="2" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n"/>
+      <c r="B159" s="2" t="n"/>
+      <c r="C159" s="2" t="n"/>
+      <c r="D159" s="2" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n"/>
+      <c r="B160" s="2" t="n"/>
+      <c r="C160" s="2" t="n"/>
+      <c r="D160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n"/>
+      <c r="B161" s="2" t="n"/>
+      <c r="C161" s="2" t="n"/>
+      <c r="D161" s="2" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n"/>
+      <c r="B162" s="2" t="n"/>
+      <c r="C162" s="2" t="n"/>
+      <c r="D162" s="2" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n"/>
+      <c r="B163" s="2" t="n"/>
+      <c r="C163" s="2" t="n"/>
+      <c r="D163" s="2" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n"/>
+      <c r="B164" s="2" t="n"/>
+      <c r="C164" s="2" t="n"/>
+      <c r="D164" s="2" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n"/>
+      <c r="B165" s="2" t="n"/>
+      <c r="C165" s="2" t="n"/>
+      <c r="D165" s="2" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n"/>
+      <c r="B166" s="2" t="n"/>
+      <c r="C166" s="2" t="n"/>
+      <c r="D166" s="2" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n"/>
+      <c r="B167" s="2" t="n"/>
+      <c r="C167" s="2" t="n"/>
+      <c r="D167" s="2" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n"/>
+      <c r="B168" s="2" t="n"/>
+      <c r="C168" s="2" t="n"/>
+      <c r="D168" s="2" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n"/>
+      <c r="B169" s="2" t="n"/>
+      <c r="C169" s="2" t="n"/>
+      <c r="D169" s="2" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n"/>
+      <c r="B170" s="2" t="n"/>
+      <c r="C170" s="2" t="n"/>
+      <c r="D170" s="2" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n"/>
+      <c r="B171" s="2" t="n"/>
+      <c r="C171" s="2" t="n"/>
+      <c r="D171" s="2" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n"/>
+      <c r="B172" s="2" t="n"/>
+      <c r="C172" s="2" t="n"/>
+      <c r="D172" s="2" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n"/>
+      <c r="B173" s="2" t="n"/>
+      <c r="C173" s="2" t="n"/>
+      <c r="D173" s="2" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n"/>
+      <c r="B174" s="2" t="n"/>
+      <c r="C174" s="2" t="n"/>
+      <c r="D174" s="2" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n"/>
+      <c r="B175" s="2" t="n"/>
+      <c r="C175" s="2" t="n"/>
+      <c r="D175" s="2" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n"/>
+      <c r="B176" s="2" t="n"/>
+      <c r="C176" s="2" t="n"/>
+      <c r="D176" s="2" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n"/>
+      <c r="B177" s="2" t="n"/>
+      <c r="C177" s="2" t="n"/>
+      <c r="D177" s="2" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n"/>
+      <c r="B178" s="2" t="n"/>
+      <c r="C178" s="2" t="n"/>
+      <c r="D178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n"/>
+      <c r="B179" s="2" t="n"/>
+      <c r="C179" s="2" t="n"/>
+      <c r="D179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n"/>
+      <c r="B180" s="2" t="n"/>
+      <c r="C180" s="2" t="n"/>
+      <c r="D180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n"/>
+      <c r="B181" s="2" t="n"/>
+      <c r="C181" s="2" t="n"/>
+      <c r="D181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n"/>
+      <c r="B182" s="2" t="n"/>
+      <c r="C182" s="2" t="n"/>
+      <c r="D182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n"/>
+      <c r="B183" s="2" t="n"/>
+      <c r="C183" s="2" t="n"/>
+      <c r="D183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n"/>
+      <c r="B184" s="2" t="n"/>
+      <c r="C184" s="2" t="n"/>
+      <c r="D184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n"/>
+      <c r="B185" s="2" t="n"/>
+      <c r="C185" s="2" t="n"/>
+      <c r="D185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n"/>
+      <c r="B186" s="2" t="n"/>
+      <c r="C186" s="2" t="n"/>
+      <c r="D186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n"/>
+      <c r="B187" s="2" t="n"/>
+      <c r="C187" s="2" t="n"/>
+      <c r="D187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n"/>
+      <c r="B188" s="2" t="n"/>
+      <c r="C188" s="2" t="n"/>
+      <c r="D188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n"/>
+      <c r="B189" s="2" t="n"/>
+      <c r="C189" s="2" t="n"/>
+      <c r="D189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n"/>
+      <c r="B190" s="2" t="n"/>
+      <c r="C190" s="2" t="n"/>
+      <c r="D190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n"/>
+      <c r="B191" s="2" t="n"/>
+      <c r="C191" s="2" t="n"/>
+      <c r="D191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n"/>
+      <c r="B192" s="2" t="n"/>
+      <c r="C192" s="2" t="n"/>
+      <c r="D192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n"/>
+      <c r="B193" s="2" t="n"/>
+      <c r="C193" s="2" t="n"/>
+      <c r="D193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n"/>
+      <c r="B194" s="2" t="n"/>
+      <c r="C194" s="2" t="n"/>
+      <c r="D194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n"/>
+      <c r="B195" s="2" t="n"/>
+      <c r="C195" s="2" t="n"/>
+      <c r="D195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n"/>
+      <c r="B196" s="2" t="n"/>
+      <c r="C196" s="2" t="n"/>
+      <c r="D196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n"/>
+      <c r="B197" s="2" t="n"/>
+      <c r="C197" s="2" t="n"/>
+      <c r="D197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n"/>
+      <c r="B198" s="2" t="n"/>
+      <c r="C198" s="2" t="n"/>
+      <c r="D198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n"/>
+      <c r="B199" s="2" t="n"/>
+      <c r="C199" s="2" t="n"/>
+      <c r="D199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n"/>
+      <c r="B200" s="2" t="n"/>
+      <c r="C200" s="2" t="n"/>
+      <c r="D200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n"/>
+      <c r="B201" s="2" t="n"/>
+      <c r="C201" s="2" t="n"/>
+      <c r="D201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n"/>
+      <c r="B202" s="2" t="n"/>
+      <c r="C202" s="2" t="n"/>
+      <c r="D202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n"/>
+      <c r="B203" s="2" t="n"/>
+      <c r="C203" s="2" t="n"/>
+      <c r="D203" s="2" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n"/>
+      <c r="B204" s="2" t="n"/>
+      <c r="C204" s="2" t="n"/>
+      <c r="D204" s="2" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n"/>
+      <c r="B205" s="2" t="n"/>
+      <c r="C205" s="2" t="n"/>
+      <c r="D205" s="2" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n"/>
+      <c r="B206" s="2" t="n"/>
+      <c r="C206" s="2" t="n"/>
+      <c r="D206" s="2" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n"/>
+      <c r="B207" s="2" t="n"/>
+      <c r="C207" s="2" t="n"/>
+      <c r="D207" s="2" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n"/>
+      <c r="B208" s="2" t="n"/>
+      <c r="C208" s="2" t="n"/>
+      <c r="D208" s="2" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n"/>
+      <c r="B209" s="2" t="n"/>
+      <c r="C209" s="2" t="n"/>
+      <c r="D209" s="2" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n"/>
+      <c r="B210" s="2" t="n"/>
+      <c r="C210" s="2" t="n"/>
+      <c r="D210" s="2" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n"/>
+      <c r="B211" s="2" t="n"/>
+      <c r="C211" s="2" t="n"/>
+      <c r="D211" s="2" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n"/>
+      <c r="B212" s="2" t="n"/>
+      <c r="C212" s="2" t="n"/>
+      <c r="D212" s="2" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n"/>
+      <c r="B213" s="2" t="n"/>
+      <c r="C213" s="2" t="n"/>
+      <c r="D213" s="2" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n"/>
+      <c r="B214" s="2" t="n"/>
+      <c r="C214" s="2" t="n"/>
+      <c r="D214" s="2" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n"/>
+      <c r="B215" s="2" t="n"/>
+      <c r="C215" s="2" t="n"/>
+      <c r="D215" s="2" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n"/>
+      <c r="B216" s="2" t="n"/>
+      <c r="C216" s="2" t="n"/>
+      <c r="D216" s="2" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n"/>
+      <c r="B217" s="2" t="n"/>
+      <c r="C217" s="2" t="n"/>
+      <c r="D217" s="2" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n"/>
+      <c r="B218" s="2" t="n"/>
+      <c r="C218" s="2" t="n"/>
+      <c r="D218" s="2" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n"/>
+      <c r="B219" s="2" t="n"/>
+      <c r="C219" s="2" t="n"/>
+      <c r="D219" s="2" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n"/>
+      <c r="B220" s="2" t="n"/>
+      <c r="C220" s="2" t="n"/>
+      <c r="D220" s="2" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n"/>
+      <c r="B221" s="2" t="n"/>
+      <c r="C221" s="2" t="n"/>
+      <c r="D221" s="2" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n"/>
+      <c r="B222" s="2" t="n"/>
+      <c r="C222" s="2" t="n"/>
+      <c r="D222" s="2" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n"/>
+      <c r="B223" s="2" t="n"/>
+      <c r="C223" s="2" t="n"/>
+      <c r="D223" s="2" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n"/>
+      <c r="B224" s="2" t="n"/>
+      <c r="C224" s="2" t="n"/>
+      <c r="D224" s="2" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n"/>
+      <c r="B225" s="2" t="n"/>
+      <c r="C225" s="2" t="n"/>
+      <c r="D225" s="2" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n"/>
+      <c r="B226" s="2" t="n"/>
+      <c r="C226" s="2" t="n"/>
+      <c r="D226" s="2" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n"/>
+      <c r="B227" s="2" t="n"/>
+      <c r="C227" s="2" t="n"/>
+      <c r="D227" s="2" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n"/>
+      <c r="B228" s="2" t="n"/>
+      <c r="C228" s="2" t="n"/>
+      <c r="D228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n"/>
+      <c r="B229" s="2" t="n"/>
+      <c r="C229" s="2" t="n"/>
+      <c r="D229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n"/>
+      <c r="B230" s="2" t="n"/>
+      <c r="C230" s="2" t="n"/>
+      <c r="D230" s="2" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n"/>
+      <c r="B231" s="2" t="n"/>
+      <c r="C231" s="2" t="n"/>
+      <c r="D231" s="2" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n"/>
+      <c r="B232" s="2" t="n"/>
+      <c r="C232" s="2" t="n"/>
+      <c r="D232" s="2" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n"/>
+      <c r="B233" s="2" t="n"/>
+      <c r="C233" s="2" t="n"/>
+      <c r="D233" s="2" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n"/>
+      <c r="B234" s="2" t="n"/>
+      <c r="C234" s="2" t="n"/>
+      <c r="D234" s="2" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n"/>
+      <c r="B235" s="2" t="n"/>
+      <c r="C235" s="2" t="n"/>
+      <c r="D235" s="2" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n"/>
+      <c r="B236" s="2" t="n"/>
+      <c r="C236" s="2" t="n"/>
+      <c r="D236" s="2" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n"/>
+      <c r="B237" s="2" t="n"/>
+      <c r="C237" s="2" t="n"/>
+      <c r="D237" s="2" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n"/>
+      <c r="B238" s="2" t="n"/>
+      <c r="C238" s="2" t="n"/>
+      <c r="D238" s="2" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n"/>
+      <c r="B239" s="2" t="n"/>
+      <c r="C239" s="2" t="n"/>
+      <c r="D239" s="2" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n"/>
+      <c r="B240" s="2" t="n"/>
+      <c r="C240" s="2" t="n"/>
+      <c r="D240" s="2" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n"/>
+      <c r="B241" s="2" t="n"/>
+      <c r="C241" s="2" t="n"/>
+      <c r="D241" s="2" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n"/>
+      <c r="B242" s="2" t="n"/>
+      <c r="C242" s="2" t="n"/>
+      <c r="D242" s="2" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n"/>
+      <c r="B243" s="2" t="n"/>
+      <c r="C243" s="2" t="n"/>
+      <c r="D243" s="2" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n"/>
+      <c r="B244" s="2" t="n"/>
+      <c r="C244" s="2" t="n"/>
+      <c r="D244" s="2" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n"/>
+      <c r="B245" s="2" t="n"/>
+      <c r="C245" s="2" t="n"/>
+      <c r="D245" s="2" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n"/>
+      <c r="B246" s="2" t="n"/>
+      <c r="C246" s="2" t="n"/>
+      <c r="D246" s="2" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n"/>
+      <c r="B247" s="2" t="n"/>
+      <c r="C247" s="2" t="n"/>
+      <c r="D247" s="2" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n"/>
+      <c r="B248" s="2" t="n"/>
+      <c r="C248" s="2" t="n"/>
+      <c r="D248" s="2" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n"/>
+      <c r="B249" s="2" t="n"/>
+      <c r="C249" s="2" t="n"/>
+      <c r="D249" s="2" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n"/>
+      <c r="B250" s="2" t="n"/>
+      <c r="C250" s="2" t="n"/>
+      <c r="D250" s="2" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n"/>
+      <c r="B251" s="2" t="n"/>
+      <c r="C251" s="2" t="n"/>
+      <c r="D251" s="2" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n"/>
+      <c r="B252" s="2" t="n"/>
+      <c r="C252" s="2" t="n"/>
+      <c r="D252" s="2" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n"/>
+      <c r="B253" s="2" t="n"/>
+      <c r="C253" s="2" t="n"/>
+      <c r="D253" s="2" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n"/>
+      <c r="B254" s="2" t="n"/>
+      <c r="C254" s="2" t="n"/>
+      <c r="D254" s="2" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n"/>
+      <c r="B255" s="2" t="n"/>
+      <c r="C255" s="2" t="n"/>
+      <c r="D255" s="2" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n"/>
+      <c r="B256" s="2" t="n"/>
+      <c r="C256" s="2" t="n"/>
+      <c r="D256" s="2" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n"/>
+      <c r="B257" s="2" t="n"/>
+      <c r="C257" s="2" t="n"/>
+      <c r="D257" s="2" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n"/>
+      <c r="B258" s="2" t="n"/>
+      <c r="C258" s="2" t="n"/>
+      <c r="D258" s="2" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n"/>
+      <c r="B259" s="2" t="n"/>
+      <c r="C259" s="2" t="n"/>
+      <c r="D259" s="2" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n"/>
+      <c r="B260" s="2" t="n"/>
+      <c r="C260" s="2" t="n"/>
+      <c r="D260" s="2" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n"/>
+      <c r="B261" s="2" t="n"/>
+      <c r="C261" s="2" t="n"/>
+      <c r="D261" s="2" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n"/>
+      <c r="B262" s="2" t="n"/>
+      <c r="C262" s="2" t="n"/>
+      <c r="D262" s="2" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n"/>
+      <c r="B263" s="2" t="n"/>
+      <c r="C263" s="2" t="n"/>
+      <c r="D263" s="2" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n"/>
+      <c r="B264" s="2" t="n"/>
+      <c r="C264" s="2" t="n"/>
+      <c r="D264" s="2" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n"/>
+      <c r="B265" s="2" t="n"/>
+      <c r="C265" s="2" t="n"/>
+      <c r="D265" s="2" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="n"/>
+      <c r="B266" s="2" t="n"/>
+      <c r="C266" s="2" t="n"/>
+      <c r="D266" s="2" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n"/>
+      <c r="B267" s="2" t="n"/>
+      <c r="C267" s="2" t="n"/>
+      <c r="D267" s="2" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n"/>
+      <c r="B268" s="2" t="n"/>
+      <c r="C268" s="2" t="n"/>
+      <c r="D268" s="2" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n"/>
+      <c r="B269" s="2" t="n"/>
+      <c r="C269" s="2" t="n"/>
+      <c r="D269" s="2" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n"/>
+      <c r="B270" s="2" t="n"/>
+      <c r="C270" s="2" t="n"/>
+      <c r="D270" s="2" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n"/>
+      <c r="B271" s="2" t="n"/>
+      <c r="C271" s="2" t="n"/>
+      <c r="D271" s="2" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n"/>
+      <c r="B272" s="2" t="n"/>
+      <c r="C272" s="2" t="n"/>
+      <c r="D272" s="2" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n"/>
+      <c r="B273" s="2" t="n"/>
+      <c r="C273" s="2" t="n"/>
+      <c r="D273" s="2" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n"/>
+      <c r="B274" s="2" t="n"/>
+      <c r="C274" s="2" t="n"/>
+      <c r="D274" s="2" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n"/>
+      <c r="B275" s="2" t="n"/>
+      <c r="C275" s="2" t="n"/>
+      <c r="D275" s="2" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n"/>
+      <c r="B276" s="2" t="n"/>
+      <c r="C276" s="2" t="n"/>
+      <c r="D276" s="2" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n"/>
+      <c r="B277" s="2" t="n"/>
+      <c r="C277" s="2" t="n"/>
+      <c r="D277" s="2" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n"/>
+      <c r="B278" s="2" t="n"/>
+      <c r="C278" s="2" t="n"/>
+      <c r="D278" s="2" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n"/>
+      <c r="B279" s="2" t="n"/>
+      <c r="C279" s="2" t="n"/>
+      <c r="D279" s="2" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n"/>
+      <c r="B280" s="2" t="n"/>
+      <c r="C280" s="2" t="n"/>
+      <c r="D280" s="2" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="n"/>
+      <c r="B281" s="2" t="n"/>
+      <c r="C281" s="2" t="n"/>
+      <c r="D281" s="2" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n"/>
+      <c r="B282" s="2" t="n"/>
+      <c r="C282" s="2" t="n"/>
+      <c r="D282" s="2" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="n"/>
+      <c r="B283" s="2" t="n"/>
+      <c r="C283" s="2" t="n"/>
+      <c r="D283" s="2" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="n"/>
+      <c r="B284" s="2" t="n"/>
+      <c r="C284" s="2" t="n"/>
+      <c r="D284" s="2" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="n"/>
+      <c r="B285" s="2" t="n"/>
+      <c r="C285" s="2" t="n"/>
+      <c r="D285" s="2" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="n"/>
+      <c r="B286" s="2" t="n"/>
+      <c r="C286" s="2" t="n"/>
+      <c r="D286" s="2" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="n"/>
+      <c r="B287" s="2" t="n"/>
+      <c r="C287" s="2" t="n"/>
+      <c r="D287" s="2" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n"/>
+      <c r="B288" s="2" t="n"/>
+      <c r="C288" s="2" t="n"/>
+      <c r="D288" s="2" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="n"/>
+      <c r="B289" s="2" t="n"/>
+      <c r="C289" s="2" t="n"/>
+      <c r="D289" s="2" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n"/>
+      <c r="B290" s="2" t="n"/>
+      <c r="C290" s="2" t="n"/>
+      <c r="D290" s="2" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="n"/>
+      <c r="B291" s="2" t="n"/>
+      <c r="C291" s="2" t="n"/>
+      <c r="D291" s="2" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="n"/>
+      <c r="B292" s="2" t="n"/>
+      <c r="C292" s="2" t="n"/>
+      <c r="D292" s="2" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="n"/>
+      <c r="B293" s="2" t="n"/>
+      <c r="C293" s="2" t="n"/>
+      <c r="D293" s="2" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="n"/>
+      <c r="B294" s="2" t="n"/>
+      <c r="C294" s="2" t="n"/>
+      <c r="D294" s="2" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="n"/>
+      <c r="B295" s="2" t="n"/>
+      <c r="C295" s="2" t="n"/>
+      <c r="D295" s="2" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="n"/>
+      <c r="B296" s="2" t="n"/>
+      <c r="C296" s="2" t="n"/>
+      <c r="D296" s="2" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="n"/>
+      <c r="B297" s="2" t="n"/>
+      <c r="C297" s="2" t="n"/>
+      <c r="D297" s="2" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="n"/>
+      <c r="B298" s="2" t="n"/>
+      <c r="C298" s="2" t="n"/>
+      <c r="D298" s="2" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="n"/>
+      <c r="B299" s="2" t="n"/>
+      <c r="C299" s="2" t="n"/>
+      <c r="D299" s="2" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="n"/>
+      <c r="B300" s="2" t="n"/>
+      <c r="C300" s="2" t="n"/>
+      <c r="D300" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:D300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt datum" error="Skriv ett datum som ÅÅÅÅ-MM-DD, t.ex. 2026-11-03." prompt="Datum, t.ex. 2026-11-03. Lämna tomt för ingen gräns." type="date" operator="between">
+      <formula1>DATE(2000,1,1)</formula1>
+      <formula2>DATE(2100,12,31)</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(#28): show news from the Anslag tab on the start page
A Typ column splits the Anslag tab into banner notices (empty or Anslag)
and news (Nyhet). News shows in a "Nyheter" section under "Träning idag",
newest Visa från first, with an optional Rubrik headline. Unknown types
are skipped so a typo never becomes a red banner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -11291,13 +11291,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D300"/>
+  <dimension ref="A1:G300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11321,6 +11324,21 @@
           <t>Visa till</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Rubrik (EN)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -11343,1800 +11361,2724 @@
           <t>2026-11-03</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Anslag</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Exempel: Vi startar en ny nybörjargrupp i januari. Hör av dig till en tränare.</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Example: We are starting a new beginner group in January. Get in touch with a coach.</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Nyhet</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Exempel: Ny nybörjargrupp</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Example: New beginner group</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
       <c r="B19" s="2" t="n"/>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
       <c r="B29" s="2" t="n"/>
       <c r="C29" s="2" t="n"/>
       <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
       <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="n"/>
       <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
       <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="n"/>
       <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="n"/>
       <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="n"/>
       <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
       <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="n"/>
       <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
       <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
       <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="n"/>
       <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
       <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
       <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="n"/>
       <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
       <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="n"/>
       <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
       <c r="B58" s="2" t="n"/>
       <c r="C58" s="2" t="n"/>
       <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="n"/>
       <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n"/>
       <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
       <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
       <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="n"/>
       <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
       <c r="B67" s="2" t="n"/>
       <c r="C67" s="2" t="n"/>
       <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="n"/>
       <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="2" t="n"/>
       <c r="C69" s="2" t="n"/>
       <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="n"/>
       <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="n"/>
       <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
       <c r="B72" s="2" t="n"/>
       <c r="C72" s="2" t="n"/>
       <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="n"/>
       <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="n"/>
       <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="2" t="n"/>
       <c r="C75" s="2" t="n"/>
       <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
       <c r="B76" s="2" t="n"/>
       <c r="C76" s="2" t="n"/>
       <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
       <c r="B77" s="2" t="n"/>
       <c r="C77" s="2" t="n"/>
       <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
       <c r="B78" s="2" t="n"/>
       <c r="C78" s="2" t="n"/>
       <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
       <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="2" t="n"/>
       <c r="C80" s="2" t="n"/>
       <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
       <c r="B81" s="2" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
       <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="n"/>
       <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="2" t="n"/>
       <c r="C83" s="2" t="n"/>
       <c r="D83" s="2" t="n"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
       <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
       <c r="B85" s="2" t="n"/>
       <c r="C85" s="2" t="n"/>
       <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n"/>
       <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
       <c r="B87" s="2" t="n"/>
       <c r="C87" s="2" t="n"/>
       <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
       <c r="B88" s="2" t="n"/>
       <c r="C88" s="2" t="n"/>
       <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
       <c r="B89" s="2" t="n"/>
       <c r="C89" s="2" t="n"/>
       <c r="D89" s="2" t="n"/>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
       <c r="B90" s="2" t="n"/>
       <c r="C90" s="2" t="n"/>
       <c r="D90" s="2" t="n"/>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
       <c r="B91" s="2" t="n"/>
       <c r="C91" s="2" t="n"/>
       <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
       <c r="B92" s="2" t="n"/>
       <c r="C92" s="2" t="n"/>
       <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="2" t="n"/>
       <c r="C93" s="2" t="n"/>
       <c r="D93" s="2" t="n"/>
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="2" t="n"/>
+      <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
       <c r="B94" s="2" t="n"/>
       <c r="C94" s="2" t="n"/>
       <c r="D94" s="2" t="n"/>
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="2" t="n"/>
+      <c r="G94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
       <c r="B95" s="2" t="n"/>
       <c r="C95" s="2" t="n"/>
       <c r="D95" s="2" t="n"/>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="n"/>
+      <c r="G95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
       <c r="B96" s="2" t="n"/>
       <c r="C96" s="2" t="n"/>
       <c r="D96" s="2" t="n"/>
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="2" t="n"/>
+      <c r="G96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
       <c r="B97" s="2" t="n"/>
       <c r="C97" s="2" t="n"/>
       <c r="D97" s="2" t="n"/>
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="2" t="n"/>
+      <c r="G97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
       <c r="B98" s="2" t="n"/>
       <c r="C98" s="2" t="n"/>
       <c r="D98" s="2" t="n"/>
+      <c r="E98" s="2" t="n"/>
+      <c r="F98" s="2" t="n"/>
+      <c r="G98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
       <c r="B99" s="2" t="n"/>
       <c r="C99" s="2" t="n"/>
       <c r="D99" s="2" t="n"/>
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="2" t="n"/>
+      <c r="G99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
       <c r="B100" s="2" t="n"/>
       <c r="C100" s="2" t="n"/>
       <c r="D100" s="2" t="n"/>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="n"/>
+      <c r="G100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
       <c r="B101" s="2" t="n"/>
       <c r="C101" s="2" t="n"/>
       <c r="D101" s="2" t="n"/>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="n"/>
+      <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
       <c r="B102" s="2" t="n"/>
       <c r="C102" s="2" t="n"/>
       <c r="D102" s="2" t="n"/>
+      <c r="E102" s="2" t="n"/>
+      <c r="F102" s="2" t="n"/>
+      <c r="G102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
       <c r="B103" s="2" t="n"/>
       <c r="C103" s="2" t="n"/>
       <c r="D103" s="2" t="n"/>
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="2" t="n"/>
+      <c r="G103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
       <c r="B104" s="2" t="n"/>
       <c r="C104" s="2" t="n"/>
       <c r="D104" s="2" t="n"/>
+      <c r="E104" s="2" t="n"/>
+      <c r="F104" s="2" t="n"/>
+      <c r="G104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
       <c r="B105" s="2" t="n"/>
       <c r="C105" s="2" t="n"/>
       <c r="D105" s="2" t="n"/>
+      <c r="E105" s="2" t="n"/>
+      <c r="F105" s="2" t="n"/>
+      <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
       <c r="B106" s="2" t="n"/>
       <c r="C106" s="2" t="n"/>
       <c r="D106" s="2" t="n"/>
+      <c r="E106" s="2" t="n"/>
+      <c r="F106" s="2" t="n"/>
+      <c r="G106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
       <c r="B107" s="2" t="n"/>
       <c r="C107" s="2" t="n"/>
       <c r="D107" s="2" t="n"/>
+      <c r="E107" s="2" t="n"/>
+      <c r="F107" s="2" t="n"/>
+      <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
       <c r="B108" s="2" t="n"/>
       <c r="C108" s="2" t="n"/>
       <c r="D108" s="2" t="n"/>
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="n"/>
+      <c r="G108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
       <c r="B109" s="2" t="n"/>
       <c r="C109" s="2" t="n"/>
       <c r="D109" s="2" t="n"/>
+      <c r="E109" s="2" t="n"/>
+      <c r="F109" s="2" t="n"/>
+      <c r="G109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
       <c r="B110" s="2" t="n"/>
       <c r="C110" s="2" t="n"/>
       <c r="D110" s="2" t="n"/>
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="n"/>
+      <c r="G110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
       <c r="B111" s="2" t="n"/>
       <c r="C111" s="2" t="n"/>
       <c r="D111" s="2" t="n"/>
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="n"/>
+      <c r="G111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
       <c r="B112" s="2" t="n"/>
       <c r="C112" s="2" t="n"/>
       <c r="D112" s="2" t="n"/>
+      <c r="E112" s="2" t="n"/>
+      <c r="F112" s="2" t="n"/>
+      <c r="G112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
       <c r="B113" s="2" t="n"/>
       <c r="C113" s="2" t="n"/>
       <c r="D113" s="2" t="n"/>
+      <c r="E113" s="2" t="n"/>
+      <c r="F113" s="2" t="n"/>
+      <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
       <c r="B114" s="2" t="n"/>
       <c r="C114" s="2" t="n"/>
       <c r="D114" s="2" t="n"/>
+      <c r="E114" s="2" t="n"/>
+      <c r="F114" s="2" t="n"/>
+      <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
       <c r="B115" s="2" t="n"/>
       <c r="C115" s="2" t="n"/>
       <c r="D115" s="2" t="n"/>
+      <c r="E115" s="2" t="n"/>
+      <c r="F115" s="2" t="n"/>
+      <c r="G115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
       <c r="B116" s="2" t="n"/>
       <c r="C116" s="2" t="n"/>
       <c r="D116" s="2" t="n"/>
+      <c r="E116" s="2" t="n"/>
+      <c r="F116" s="2" t="n"/>
+      <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
       <c r="B117" s="2" t="n"/>
       <c r="C117" s="2" t="n"/>
       <c r="D117" s="2" t="n"/>
+      <c r="E117" s="2" t="n"/>
+      <c r="F117" s="2" t="n"/>
+      <c r="G117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
       <c r="B118" s="2" t="n"/>
       <c r="C118" s="2" t="n"/>
       <c r="D118" s="2" t="n"/>
+      <c r="E118" s="2" t="n"/>
+      <c r="F118" s="2" t="n"/>
+      <c r="G118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
       <c r="B119" s="2" t="n"/>
       <c r="C119" s="2" t="n"/>
       <c r="D119" s="2" t="n"/>
+      <c r="E119" s="2" t="n"/>
+      <c r="F119" s="2" t="n"/>
+      <c r="G119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
       <c r="B120" s="2" t="n"/>
       <c r="C120" s="2" t="n"/>
       <c r="D120" s="2" t="n"/>
+      <c r="E120" s="2" t="n"/>
+      <c r="F120" s="2" t="n"/>
+      <c r="G120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
       <c r="B121" s="2" t="n"/>
       <c r="C121" s="2" t="n"/>
       <c r="D121" s="2" t="n"/>
+      <c r="E121" s="2" t="n"/>
+      <c r="F121" s="2" t="n"/>
+      <c r="G121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
       <c r="B122" s="2" t="n"/>
       <c r="C122" s="2" t="n"/>
       <c r="D122" s="2" t="n"/>
+      <c r="E122" s="2" t="n"/>
+      <c r="F122" s="2" t="n"/>
+      <c r="G122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
       <c r="B123" s="2" t="n"/>
       <c r="C123" s="2" t="n"/>
       <c r="D123" s="2" t="n"/>
+      <c r="E123" s="2" t="n"/>
+      <c r="F123" s="2" t="n"/>
+      <c r="G123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
       <c r="B124" s="2" t="n"/>
       <c r="C124" s="2" t="n"/>
       <c r="D124" s="2" t="n"/>
+      <c r="E124" s="2" t="n"/>
+      <c r="F124" s="2" t="n"/>
+      <c r="G124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
       <c r="B125" s="2" t="n"/>
       <c r="C125" s="2" t="n"/>
       <c r="D125" s="2" t="n"/>
+      <c r="E125" s="2" t="n"/>
+      <c r="F125" s="2" t="n"/>
+      <c r="G125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
       <c r="B126" s="2" t="n"/>
       <c r="C126" s="2" t="n"/>
       <c r="D126" s="2" t="n"/>
+      <c r="E126" s="2" t="n"/>
+      <c r="F126" s="2" t="n"/>
+      <c r="G126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
       <c r="B127" s="2" t="n"/>
       <c r="C127" s="2" t="n"/>
       <c r="D127" s="2" t="n"/>
+      <c r="E127" s="2" t="n"/>
+      <c r="F127" s="2" t="n"/>
+      <c r="G127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
       <c r="B128" s="2" t="n"/>
       <c r="C128" s="2" t="n"/>
       <c r="D128" s="2" t="n"/>
+      <c r="E128" s="2" t="n"/>
+      <c r="F128" s="2" t="n"/>
+      <c r="G128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
       <c r="B129" s="2" t="n"/>
       <c r="C129" s="2" t="n"/>
       <c r="D129" s="2" t="n"/>
+      <c r="E129" s="2" t="n"/>
+      <c r="F129" s="2" t="n"/>
+      <c r="G129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
       <c r="B130" s="2" t="n"/>
       <c r="C130" s="2" t="n"/>
       <c r="D130" s="2" t="n"/>
+      <c r="E130" s="2" t="n"/>
+      <c r="F130" s="2" t="n"/>
+      <c r="G130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
       <c r="B131" s="2" t="n"/>
       <c r="C131" s="2" t="n"/>
       <c r="D131" s="2" t="n"/>
+      <c r="E131" s="2" t="n"/>
+      <c r="F131" s="2" t="n"/>
+      <c r="G131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
       <c r="B132" s="2" t="n"/>
       <c r="C132" s="2" t="n"/>
       <c r="D132" s="2" t="n"/>
+      <c r="E132" s="2" t="n"/>
+      <c r="F132" s="2" t="n"/>
+      <c r="G132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
       <c r="B133" s="2" t="n"/>
       <c r="C133" s="2" t="n"/>
       <c r="D133" s="2" t="n"/>
+      <c r="E133" s="2" t="n"/>
+      <c r="F133" s="2" t="n"/>
+      <c r="G133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
       <c r="B134" s="2" t="n"/>
       <c r="C134" s="2" t="n"/>
       <c r="D134" s="2" t="n"/>
+      <c r="E134" s="2" t="n"/>
+      <c r="F134" s="2" t="n"/>
+      <c r="G134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
       <c r="B135" s="2" t="n"/>
       <c r="C135" s="2" t="n"/>
       <c r="D135" s="2" t="n"/>
+      <c r="E135" s="2" t="n"/>
+      <c r="F135" s="2" t="n"/>
+      <c r="G135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
       <c r="B136" s="2" t="n"/>
       <c r="C136" s="2" t="n"/>
       <c r="D136" s="2" t="n"/>
+      <c r="E136" s="2" t="n"/>
+      <c r="F136" s="2" t="n"/>
+      <c r="G136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
       <c r="B137" s="2" t="n"/>
       <c r="C137" s="2" t="n"/>
       <c r="D137" s="2" t="n"/>
+      <c r="E137" s="2" t="n"/>
+      <c r="F137" s="2" t="n"/>
+      <c r="G137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
       <c r="B138" s="2" t="n"/>
       <c r="C138" s="2" t="n"/>
       <c r="D138" s="2" t="n"/>
+      <c r="E138" s="2" t="n"/>
+      <c r="F138" s="2" t="n"/>
+      <c r="G138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
       <c r="B139" s="2" t="n"/>
       <c r="C139" s="2" t="n"/>
       <c r="D139" s="2" t="n"/>
+      <c r="E139" s="2" t="n"/>
+      <c r="F139" s="2" t="n"/>
+      <c r="G139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
       <c r="B140" s="2" t="n"/>
       <c r="C140" s="2" t="n"/>
       <c r="D140" s="2" t="n"/>
+      <c r="E140" s="2" t="n"/>
+      <c r="F140" s="2" t="n"/>
+      <c r="G140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
       <c r="B141" s="2" t="n"/>
       <c r="C141" s="2" t="n"/>
       <c r="D141" s="2" t="n"/>
+      <c r="E141" s="2" t="n"/>
+      <c r="F141" s="2" t="n"/>
+      <c r="G141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
       <c r="B142" s="2" t="n"/>
       <c r="C142" s="2" t="n"/>
       <c r="D142" s="2" t="n"/>
+      <c r="E142" s="2" t="n"/>
+      <c r="F142" s="2" t="n"/>
+      <c r="G142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
       <c r="B143" s="2" t="n"/>
       <c r="C143" s="2" t="n"/>
       <c r="D143" s="2" t="n"/>
+      <c r="E143" s="2" t="n"/>
+      <c r="F143" s="2" t="n"/>
+      <c r="G143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
       <c r="B144" s="2" t="n"/>
       <c r="C144" s="2" t="n"/>
       <c r="D144" s="2" t="n"/>
+      <c r="E144" s="2" t="n"/>
+      <c r="F144" s="2" t="n"/>
+      <c r="G144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
       <c r="B145" s="2" t="n"/>
       <c r="C145" s="2" t="n"/>
       <c r="D145" s="2" t="n"/>
+      <c r="E145" s="2" t="n"/>
+      <c r="F145" s="2" t="n"/>
+      <c r="G145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
       <c r="B146" s="2" t="n"/>
       <c r="C146" s="2" t="n"/>
       <c r="D146" s="2" t="n"/>
+      <c r="E146" s="2" t="n"/>
+      <c r="F146" s="2" t="n"/>
+      <c r="G146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
       <c r="B147" s="2" t="n"/>
       <c r="C147" s="2" t="n"/>
       <c r="D147" s="2" t="n"/>
+      <c r="E147" s="2" t="n"/>
+      <c r="F147" s="2" t="n"/>
+      <c r="G147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
       <c r="B148" s="2" t="n"/>
       <c r="C148" s="2" t="n"/>
       <c r="D148" s="2" t="n"/>
+      <c r="E148" s="2" t="n"/>
+      <c r="F148" s="2" t="n"/>
+      <c r="G148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
       <c r="B149" s="2" t="n"/>
       <c r="C149" s="2" t="n"/>
       <c r="D149" s="2" t="n"/>
+      <c r="E149" s="2" t="n"/>
+      <c r="F149" s="2" t="n"/>
+      <c r="G149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
       <c r="B150" s="2" t="n"/>
       <c r="C150" s="2" t="n"/>
       <c r="D150" s="2" t="n"/>
+      <c r="E150" s="2" t="n"/>
+      <c r="F150" s="2" t="n"/>
+      <c r="G150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
       <c r="B151" s="2" t="n"/>
       <c r="C151" s="2" t="n"/>
       <c r="D151" s="2" t="n"/>
+      <c r="E151" s="2" t="n"/>
+      <c r="F151" s="2" t="n"/>
+      <c r="G151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
       <c r="B152" s="2" t="n"/>
       <c r="C152" s="2" t="n"/>
       <c r="D152" s="2" t="n"/>
+      <c r="E152" s="2" t="n"/>
+      <c r="F152" s="2" t="n"/>
+      <c r="G152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
       <c r="B153" s="2" t="n"/>
       <c r="C153" s="2" t="n"/>
       <c r="D153" s="2" t="n"/>
+      <c r="E153" s="2" t="n"/>
+      <c r="F153" s="2" t="n"/>
+      <c r="G153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
       <c r="B154" s="2" t="n"/>
       <c r="C154" s="2" t="n"/>
       <c r="D154" s="2" t="n"/>
+      <c r="E154" s="2" t="n"/>
+      <c r="F154" s="2" t="n"/>
+      <c r="G154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
       <c r="B155" s="2" t="n"/>
       <c r="C155" s="2" t="n"/>
       <c r="D155" s="2" t="n"/>
+      <c r="E155" s="2" t="n"/>
+      <c r="F155" s="2" t="n"/>
+      <c r="G155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
       <c r="B156" s="2" t="n"/>
       <c r="C156" s="2" t="n"/>
       <c r="D156" s="2" t="n"/>
+      <c r="E156" s="2" t="n"/>
+      <c r="F156" s="2" t="n"/>
+      <c r="G156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
       <c r="B157" s="2" t="n"/>
       <c r="C157" s="2" t="n"/>
       <c r="D157" s="2" t="n"/>
+      <c r="E157" s="2" t="n"/>
+      <c r="F157" s="2" t="n"/>
+      <c r="G157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
       <c r="B158" s="2" t="n"/>
       <c r="C158" s="2" t="n"/>
       <c r="D158" s="2" t="n"/>
+      <c r="E158" s="2" t="n"/>
+      <c r="F158" s="2" t="n"/>
+      <c r="G158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
       <c r="B159" s="2" t="n"/>
       <c r="C159" s="2" t="n"/>
       <c r="D159" s="2" t="n"/>
+      <c r="E159" s="2" t="n"/>
+      <c r="F159" s="2" t="n"/>
+      <c r="G159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
       <c r="B160" s="2" t="n"/>
       <c r="C160" s="2" t="n"/>
       <c r="D160" s="2" t="n"/>
+      <c r="E160" s="2" t="n"/>
+      <c r="F160" s="2" t="n"/>
+      <c r="G160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
       <c r="B161" s="2" t="n"/>
       <c r="C161" s="2" t="n"/>
       <c r="D161" s="2" t="n"/>
+      <c r="E161" s="2" t="n"/>
+      <c r="F161" s="2" t="n"/>
+      <c r="G161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
       <c r="B162" s="2" t="n"/>
       <c r="C162" s="2" t="n"/>
       <c r="D162" s="2" t="n"/>
+      <c r="E162" s="2" t="n"/>
+      <c r="F162" s="2" t="n"/>
+      <c r="G162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
       <c r="B163" s="2" t="n"/>
       <c r="C163" s="2" t="n"/>
       <c r="D163" s="2" t="n"/>
+      <c r="E163" s="2" t="n"/>
+      <c r="F163" s="2" t="n"/>
+      <c r="G163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
       <c r="B164" s="2" t="n"/>
       <c r="C164" s="2" t="n"/>
       <c r="D164" s="2" t="n"/>
+      <c r="E164" s="2" t="n"/>
+      <c r="F164" s="2" t="n"/>
+      <c r="G164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
       <c r="B165" s="2" t="n"/>
       <c r="C165" s="2" t="n"/>
       <c r="D165" s="2" t="n"/>
+      <c r="E165" s="2" t="n"/>
+      <c r="F165" s="2" t="n"/>
+      <c r="G165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
       <c r="B166" s="2" t="n"/>
       <c r="C166" s="2" t="n"/>
       <c r="D166" s="2" t="n"/>
+      <c r="E166" s="2" t="n"/>
+      <c r="F166" s="2" t="n"/>
+      <c r="G166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
       <c r="B167" s="2" t="n"/>
       <c r="C167" s="2" t="n"/>
       <c r="D167" s="2" t="n"/>
+      <c r="E167" s="2" t="n"/>
+      <c r="F167" s="2" t="n"/>
+      <c r="G167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
       <c r="B168" s="2" t="n"/>
       <c r="C168" s="2" t="n"/>
       <c r="D168" s="2" t="n"/>
+      <c r="E168" s="2" t="n"/>
+      <c r="F168" s="2" t="n"/>
+      <c r="G168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
       <c r="B169" s="2" t="n"/>
       <c r="C169" s="2" t="n"/>
       <c r="D169" s="2" t="n"/>
+      <c r="E169" s="2" t="n"/>
+      <c r="F169" s="2" t="n"/>
+      <c r="G169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
       <c r="B170" s="2" t="n"/>
       <c r="C170" s="2" t="n"/>
       <c r="D170" s="2" t="n"/>
+      <c r="E170" s="2" t="n"/>
+      <c r="F170" s="2" t="n"/>
+      <c r="G170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
       <c r="B171" s="2" t="n"/>
       <c r="C171" s="2" t="n"/>
       <c r="D171" s="2" t="n"/>
+      <c r="E171" s="2" t="n"/>
+      <c r="F171" s="2" t="n"/>
+      <c r="G171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
       <c r="B172" s="2" t="n"/>
       <c r="C172" s="2" t="n"/>
       <c r="D172" s="2" t="n"/>
+      <c r="E172" s="2" t="n"/>
+      <c r="F172" s="2" t="n"/>
+      <c r="G172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
       <c r="B173" s="2" t="n"/>
       <c r="C173" s="2" t="n"/>
       <c r="D173" s="2" t="n"/>
+      <c r="E173" s="2" t="n"/>
+      <c r="F173" s="2" t="n"/>
+      <c r="G173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
       <c r="B174" s="2" t="n"/>
       <c r="C174" s="2" t="n"/>
       <c r="D174" s="2" t="n"/>
+      <c r="E174" s="2" t="n"/>
+      <c r="F174" s="2" t="n"/>
+      <c r="G174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
       <c r="B175" s="2" t="n"/>
       <c r="C175" s="2" t="n"/>
       <c r="D175" s="2" t="n"/>
+      <c r="E175" s="2" t="n"/>
+      <c r="F175" s="2" t="n"/>
+      <c r="G175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
       <c r="B176" s="2" t="n"/>
       <c r="C176" s="2" t="n"/>
       <c r="D176" s="2" t="n"/>
+      <c r="E176" s="2" t="n"/>
+      <c r="F176" s="2" t="n"/>
+      <c r="G176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
       <c r="B177" s="2" t="n"/>
       <c r="C177" s="2" t="n"/>
       <c r="D177" s="2" t="n"/>
+      <c r="E177" s="2" t="n"/>
+      <c r="F177" s="2" t="n"/>
+      <c r="G177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
       <c r="B178" s="2" t="n"/>
       <c r="C178" s="2" t="n"/>
       <c r="D178" s="2" t="n"/>
+      <c r="E178" s="2" t="n"/>
+      <c r="F178" s="2" t="n"/>
+      <c r="G178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
       <c r="B179" s="2" t="n"/>
       <c r="C179" s="2" t="n"/>
       <c r="D179" s="2" t="n"/>
+      <c r="E179" s="2" t="n"/>
+      <c r="F179" s="2" t="n"/>
+      <c r="G179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
       <c r="B180" s="2" t="n"/>
       <c r="C180" s="2" t="n"/>
       <c r="D180" s="2" t="n"/>
+      <c r="E180" s="2" t="n"/>
+      <c r="F180" s="2" t="n"/>
+      <c r="G180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
       <c r="B181" s="2" t="n"/>
       <c r="C181" s="2" t="n"/>
       <c r="D181" s="2" t="n"/>
+      <c r="E181" s="2" t="n"/>
+      <c r="F181" s="2" t="n"/>
+      <c r="G181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
       <c r="B182" s="2" t="n"/>
       <c r="C182" s="2" t="n"/>
       <c r="D182" s="2" t="n"/>
+      <c r="E182" s="2" t="n"/>
+      <c r="F182" s="2" t="n"/>
+      <c r="G182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
       <c r="B183" s="2" t="n"/>
       <c r="C183" s="2" t="n"/>
       <c r="D183" s="2" t="n"/>
+      <c r="E183" s="2" t="n"/>
+      <c r="F183" s="2" t="n"/>
+      <c r="G183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
       <c r="B184" s="2" t="n"/>
       <c r="C184" s="2" t="n"/>
       <c r="D184" s="2" t="n"/>
+      <c r="E184" s="2" t="n"/>
+      <c r="F184" s="2" t="n"/>
+      <c r="G184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
       <c r="B185" s="2" t="n"/>
       <c r="C185" s="2" t="n"/>
       <c r="D185" s="2" t="n"/>
+      <c r="E185" s="2" t="n"/>
+      <c r="F185" s="2" t="n"/>
+      <c r="G185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
       <c r="B186" s="2" t="n"/>
       <c r="C186" s="2" t="n"/>
       <c r="D186" s="2" t="n"/>
+      <c r="E186" s="2" t="n"/>
+      <c r="F186" s="2" t="n"/>
+      <c r="G186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
       <c r="B187" s="2" t="n"/>
       <c r="C187" s="2" t="n"/>
       <c r="D187" s="2" t="n"/>
+      <c r="E187" s="2" t="n"/>
+      <c r="F187" s="2" t="n"/>
+      <c r="G187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
       <c r="B188" s="2" t="n"/>
       <c r="C188" s="2" t="n"/>
       <c r="D188" s="2" t="n"/>
+      <c r="E188" s="2" t="n"/>
+      <c r="F188" s="2" t="n"/>
+      <c r="G188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
       <c r="B189" s="2" t="n"/>
       <c r="C189" s="2" t="n"/>
       <c r="D189" s="2" t="n"/>
+      <c r="E189" s="2" t="n"/>
+      <c r="F189" s="2" t="n"/>
+      <c r="G189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
       <c r="B190" s="2" t="n"/>
       <c r="C190" s="2" t="n"/>
       <c r="D190" s="2" t="n"/>
+      <c r="E190" s="2" t="n"/>
+      <c r="F190" s="2" t="n"/>
+      <c r="G190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
       <c r="B191" s="2" t="n"/>
       <c r="C191" s="2" t="n"/>
       <c r="D191" s="2" t="n"/>
+      <c r="E191" s="2" t="n"/>
+      <c r="F191" s="2" t="n"/>
+      <c r="G191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
       <c r="B192" s="2" t="n"/>
       <c r="C192" s="2" t="n"/>
       <c r="D192" s="2" t="n"/>
+      <c r="E192" s="2" t="n"/>
+      <c r="F192" s="2" t="n"/>
+      <c r="G192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
       <c r="B193" s="2" t="n"/>
       <c r="C193" s="2" t="n"/>
       <c r="D193" s="2" t="n"/>
+      <c r="E193" s="2" t="n"/>
+      <c r="F193" s="2" t="n"/>
+      <c r="G193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
       <c r="B194" s="2" t="n"/>
       <c r="C194" s="2" t="n"/>
       <c r="D194" s="2" t="n"/>
+      <c r="E194" s="2" t="n"/>
+      <c r="F194" s="2" t="n"/>
+      <c r="G194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
       <c r="B195" s="2" t="n"/>
       <c r="C195" s="2" t="n"/>
       <c r="D195" s="2" t="n"/>
+      <c r="E195" s="2" t="n"/>
+      <c r="F195" s="2" t="n"/>
+      <c r="G195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
       <c r="B196" s="2" t="n"/>
       <c r="C196" s="2" t="n"/>
       <c r="D196" s="2" t="n"/>
+      <c r="E196" s="2" t="n"/>
+      <c r="F196" s="2" t="n"/>
+      <c r="G196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
       <c r="B197" s="2" t="n"/>
       <c r="C197" s="2" t="n"/>
       <c r="D197" s="2" t="n"/>
+      <c r="E197" s="2" t="n"/>
+      <c r="F197" s="2" t="n"/>
+      <c r="G197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
       <c r="B198" s="2" t="n"/>
       <c r="C198" s="2" t="n"/>
       <c r="D198" s="2" t="n"/>
+      <c r="E198" s="2" t="n"/>
+      <c r="F198" s="2" t="n"/>
+      <c r="G198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
       <c r="B199" s="2" t="n"/>
       <c r="C199" s="2" t="n"/>
       <c r="D199" s="2" t="n"/>
+      <c r="E199" s="2" t="n"/>
+      <c r="F199" s="2" t="n"/>
+      <c r="G199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
       <c r="B200" s="2" t="n"/>
       <c r="C200" s="2" t="n"/>
       <c r="D200" s="2" t="n"/>
+      <c r="E200" s="2" t="n"/>
+      <c r="F200" s="2" t="n"/>
+      <c r="G200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
       <c r="B201" s="2" t="n"/>
       <c r="C201" s="2" t="n"/>
       <c r="D201" s="2" t="n"/>
+      <c r="E201" s="2" t="n"/>
+      <c r="F201" s="2" t="n"/>
+      <c r="G201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n"/>
       <c r="B202" s="2" t="n"/>
       <c r="C202" s="2" t="n"/>
       <c r="D202" s="2" t="n"/>
+      <c r="E202" s="2" t="n"/>
+      <c r="F202" s="2" t="n"/>
+      <c r="G202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n"/>
       <c r="B203" s="2" t="n"/>
       <c r="C203" s="2" t="n"/>
       <c r="D203" s="2" t="n"/>
+      <c r="E203" s="2" t="n"/>
+      <c r="F203" s="2" t="n"/>
+      <c r="G203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n"/>
       <c r="B204" s="2" t="n"/>
       <c r="C204" s="2" t="n"/>
       <c r="D204" s="2" t="n"/>
+      <c r="E204" s="2" t="n"/>
+      <c r="F204" s="2" t="n"/>
+      <c r="G204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
       <c r="B205" s="2" t="n"/>
       <c r="C205" s="2" t="n"/>
       <c r="D205" s="2" t="n"/>
+      <c r="E205" s="2" t="n"/>
+      <c r="F205" s="2" t="n"/>
+      <c r="G205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n"/>
       <c r="B206" s="2" t="n"/>
       <c r="C206" s="2" t="n"/>
       <c r="D206" s="2" t="n"/>
+      <c r="E206" s="2" t="n"/>
+      <c r="F206" s="2" t="n"/>
+      <c r="G206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
       <c r="B207" s="2" t="n"/>
       <c r="C207" s="2" t="n"/>
       <c r="D207" s="2" t="n"/>
+      <c r="E207" s="2" t="n"/>
+      <c r="F207" s="2" t="n"/>
+      <c r="G207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
       <c r="B208" s="2" t="n"/>
       <c r="C208" s="2" t="n"/>
       <c r="D208" s="2" t="n"/>
+      <c r="E208" s="2" t="n"/>
+      <c r="F208" s="2" t="n"/>
+      <c r="G208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n"/>
       <c r="B209" s="2" t="n"/>
       <c r="C209" s="2" t="n"/>
       <c r="D209" s="2" t="n"/>
+      <c r="E209" s="2" t="n"/>
+      <c r="F209" s="2" t="n"/>
+      <c r="G209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
       <c r="B210" s="2" t="n"/>
       <c r="C210" s="2" t="n"/>
       <c r="D210" s="2" t="n"/>
+      <c r="E210" s="2" t="n"/>
+      <c r="F210" s="2" t="n"/>
+      <c r="G210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n"/>
       <c r="B211" s="2" t="n"/>
       <c r="C211" s="2" t="n"/>
       <c r="D211" s="2" t="n"/>
+      <c r="E211" s="2" t="n"/>
+      <c r="F211" s="2" t="n"/>
+      <c r="G211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
       <c r="B212" s="2" t="n"/>
       <c r="C212" s="2" t="n"/>
       <c r="D212" s="2" t="n"/>
+      <c r="E212" s="2" t="n"/>
+      <c r="F212" s="2" t="n"/>
+      <c r="G212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
       <c r="B213" s="2" t="n"/>
       <c r="C213" s="2" t="n"/>
       <c r="D213" s="2" t="n"/>
+      <c r="E213" s="2" t="n"/>
+      <c r="F213" s="2" t="n"/>
+      <c r="G213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n"/>
       <c r="B214" s="2" t="n"/>
       <c r="C214" s="2" t="n"/>
       <c r="D214" s="2" t="n"/>
+      <c r="E214" s="2" t="n"/>
+      <c r="F214" s="2" t="n"/>
+      <c r="G214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n"/>
       <c r="B215" s="2" t="n"/>
       <c r="C215" s="2" t="n"/>
       <c r="D215" s="2" t="n"/>
+      <c r="E215" s="2" t="n"/>
+      <c r="F215" s="2" t="n"/>
+      <c r="G215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n"/>
       <c r="B216" s="2" t="n"/>
       <c r="C216" s="2" t="n"/>
       <c r="D216" s="2" t="n"/>
+      <c r="E216" s="2" t="n"/>
+      <c r="F216" s="2" t="n"/>
+      <c r="G216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n"/>
       <c r="B217" s="2" t="n"/>
       <c r="C217" s="2" t="n"/>
       <c r="D217" s="2" t="n"/>
+      <c r="E217" s="2" t="n"/>
+      <c r="F217" s="2" t="n"/>
+      <c r="G217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n"/>
       <c r="B218" s="2" t="n"/>
       <c r="C218" s="2" t="n"/>
       <c r="D218" s="2" t="n"/>
+      <c r="E218" s="2" t="n"/>
+      <c r="F218" s="2" t="n"/>
+      <c r="G218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n"/>
       <c r="B219" s="2" t="n"/>
       <c r="C219" s="2" t="n"/>
       <c r="D219" s="2" t="n"/>
+      <c r="E219" s="2" t="n"/>
+      <c r="F219" s="2" t="n"/>
+      <c r="G219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n"/>
       <c r="B220" s="2" t="n"/>
       <c r="C220" s="2" t="n"/>
       <c r="D220" s="2" t="n"/>
+      <c r="E220" s="2" t="n"/>
+      <c r="F220" s="2" t="n"/>
+      <c r="G220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n"/>
       <c r="B221" s="2" t="n"/>
       <c r="C221" s="2" t="n"/>
       <c r="D221" s="2" t="n"/>
+      <c r="E221" s="2" t="n"/>
+      <c r="F221" s="2" t="n"/>
+      <c r="G221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n"/>
       <c r="B222" s="2" t="n"/>
       <c r="C222" s="2" t="n"/>
       <c r="D222" s="2" t="n"/>
+      <c r="E222" s="2" t="n"/>
+      <c r="F222" s="2" t="n"/>
+      <c r="G222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n"/>
       <c r="B223" s="2" t="n"/>
       <c r="C223" s="2" t="n"/>
       <c r="D223" s="2" t="n"/>
+      <c r="E223" s="2" t="n"/>
+      <c r="F223" s="2" t="n"/>
+      <c r="G223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n"/>
       <c r="B224" s="2" t="n"/>
       <c r="C224" s="2" t="n"/>
       <c r="D224" s="2" t="n"/>
+      <c r="E224" s="2" t="n"/>
+      <c r="F224" s="2" t="n"/>
+      <c r="G224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n"/>
       <c r="B225" s="2" t="n"/>
       <c r="C225" s="2" t="n"/>
       <c r="D225" s="2" t="n"/>
+      <c r="E225" s="2" t="n"/>
+      <c r="F225" s="2" t="n"/>
+      <c r="G225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n"/>
       <c r="B226" s="2" t="n"/>
       <c r="C226" s="2" t="n"/>
       <c r="D226" s="2" t="n"/>
+      <c r="E226" s="2" t="n"/>
+      <c r="F226" s="2" t="n"/>
+      <c r="G226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n"/>
       <c r="B227" s="2" t="n"/>
       <c r="C227" s="2" t="n"/>
       <c r="D227" s="2" t="n"/>
+      <c r="E227" s="2" t="n"/>
+      <c r="F227" s="2" t="n"/>
+      <c r="G227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n"/>
       <c r="B228" s="2" t="n"/>
       <c r="C228" s="2" t="n"/>
       <c r="D228" s="2" t="n"/>
+      <c r="E228" s="2" t="n"/>
+      <c r="F228" s="2" t="n"/>
+      <c r="G228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n"/>
       <c r="B229" s="2" t="n"/>
       <c r="C229" s="2" t="n"/>
       <c r="D229" s="2" t="n"/>
+      <c r="E229" s="2" t="n"/>
+      <c r="F229" s="2" t="n"/>
+      <c r="G229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n"/>
       <c r="B230" s="2" t="n"/>
       <c r="C230" s="2" t="n"/>
       <c r="D230" s="2" t="n"/>
+      <c r="E230" s="2" t="n"/>
+      <c r="F230" s="2" t="n"/>
+      <c r="G230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n"/>
       <c r="B231" s="2" t="n"/>
       <c r="C231" s="2" t="n"/>
       <c r="D231" s="2" t="n"/>
+      <c r="E231" s="2" t="n"/>
+      <c r="F231" s="2" t="n"/>
+      <c r="G231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n"/>
       <c r="B232" s="2" t="n"/>
       <c r="C232" s="2" t="n"/>
       <c r="D232" s="2" t="n"/>
+      <c r="E232" s="2" t="n"/>
+      <c r="F232" s="2" t="n"/>
+      <c r="G232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n"/>
       <c r="B233" s="2" t="n"/>
       <c r="C233" s="2" t="n"/>
       <c r="D233" s="2" t="n"/>
+      <c r="E233" s="2" t="n"/>
+      <c r="F233" s="2" t="n"/>
+      <c r="G233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n"/>
       <c r="B234" s="2" t="n"/>
       <c r="C234" s="2" t="n"/>
       <c r="D234" s="2" t="n"/>
+      <c r="E234" s="2" t="n"/>
+      <c r="F234" s="2" t="n"/>
+      <c r="G234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n"/>
       <c r="B235" s="2" t="n"/>
       <c r="C235" s="2" t="n"/>
       <c r="D235" s="2" t="n"/>
+      <c r="E235" s="2" t="n"/>
+      <c r="F235" s="2" t="n"/>
+      <c r="G235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n"/>
       <c r="B236" s="2" t="n"/>
       <c r="C236" s="2" t="n"/>
       <c r="D236" s="2" t="n"/>
+      <c r="E236" s="2" t="n"/>
+      <c r="F236" s="2" t="n"/>
+      <c r="G236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n"/>
       <c r="B237" s="2" t="n"/>
       <c r="C237" s="2" t="n"/>
       <c r="D237" s="2" t="n"/>
+      <c r="E237" s="2" t="n"/>
+      <c r="F237" s="2" t="n"/>
+      <c r="G237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n"/>
       <c r="B238" s="2" t="n"/>
       <c r="C238" s="2" t="n"/>
       <c r="D238" s="2" t="n"/>
+      <c r="E238" s="2" t="n"/>
+      <c r="F238" s="2" t="n"/>
+      <c r="G238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n"/>
       <c r="B239" s="2" t="n"/>
       <c r="C239" s="2" t="n"/>
       <c r="D239" s="2" t="n"/>
+      <c r="E239" s="2" t="n"/>
+      <c r="F239" s="2" t="n"/>
+      <c r="G239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n"/>
       <c r="B240" s="2" t="n"/>
       <c r="C240" s="2" t="n"/>
       <c r="D240" s="2" t="n"/>
+      <c r="E240" s="2" t="n"/>
+      <c r="F240" s="2" t="n"/>
+      <c r="G240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n"/>
       <c r="B241" s="2" t="n"/>
       <c r="C241" s="2" t="n"/>
       <c r="D241" s="2" t="n"/>
+      <c r="E241" s="2" t="n"/>
+      <c r="F241" s="2" t="n"/>
+      <c r="G241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n"/>
       <c r="B242" s="2" t="n"/>
       <c r="C242" s="2" t="n"/>
       <c r="D242" s="2" t="n"/>
+      <c r="E242" s="2" t="n"/>
+      <c r="F242" s="2" t="n"/>
+      <c r="G242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n"/>
       <c r="B243" s="2" t="n"/>
       <c r="C243" s="2" t="n"/>
       <c r="D243" s="2" t="n"/>
+      <c r="E243" s="2" t="n"/>
+      <c r="F243" s="2" t="n"/>
+      <c r="G243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n"/>
       <c r="B244" s="2" t="n"/>
       <c r="C244" s="2" t="n"/>
       <c r="D244" s="2" t="n"/>
+      <c r="E244" s="2" t="n"/>
+      <c r="F244" s="2" t="n"/>
+      <c r="G244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n"/>
       <c r="B245" s="2" t="n"/>
       <c r="C245" s="2" t="n"/>
       <c r="D245" s="2" t="n"/>
+      <c r="E245" s="2" t="n"/>
+      <c r="F245" s="2" t="n"/>
+      <c r="G245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n"/>
       <c r="B246" s="2" t="n"/>
       <c r="C246" s="2" t="n"/>
       <c r="D246" s="2" t="n"/>
+      <c r="E246" s="2" t="n"/>
+      <c r="F246" s="2" t="n"/>
+      <c r="G246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n"/>
       <c r="B247" s="2" t="n"/>
       <c r="C247" s="2" t="n"/>
       <c r="D247" s="2" t="n"/>
+      <c r="E247" s="2" t="n"/>
+      <c r="F247" s="2" t="n"/>
+      <c r="G247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n"/>
       <c r="B248" s="2" t="n"/>
       <c r="C248" s="2" t="n"/>
       <c r="D248" s="2" t="n"/>
+      <c r="E248" s="2" t="n"/>
+      <c r="F248" s="2" t="n"/>
+      <c r="G248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n"/>
       <c r="B249" s="2" t="n"/>
       <c r="C249" s="2" t="n"/>
       <c r="D249" s="2" t="n"/>
+      <c r="E249" s="2" t="n"/>
+      <c r="F249" s="2" t="n"/>
+      <c r="G249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n"/>
       <c r="B250" s="2" t="n"/>
       <c r="C250" s="2" t="n"/>
       <c r="D250" s="2" t="n"/>
+      <c r="E250" s="2" t="n"/>
+      <c r="F250" s="2" t="n"/>
+      <c r="G250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n"/>
       <c r="B251" s="2" t="n"/>
       <c r="C251" s="2" t="n"/>
       <c r="D251" s="2" t="n"/>
+      <c r="E251" s="2" t="n"/>
+      <c r="F251" s="2" t="n"/>
+      <c r="G251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n"/>
       <c r="B252" s="2" t="n"/>
       <c r="C252" s="2" t="n"/>
       <c r="D252" s="2" t="n"/>
+      <c r="E252" s="2" t="n"/>
+      <c r="F252" s="2" t="n"/>
+      <c r="G252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n"/>
       <c r="B253" s="2" t="n"/>
       <c r="C253" s="2" t="n"/>
       <c r="D253" s="2" t="n"/>
+      <c r="E253" s="2" t="n"/>
+      <c r="F253" s="2" t="n"/>
+      <c r="G253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n"/>
       <c r="B254" s="2" t="n"/>
       <c r="C254" s="2" t="n"/>
       <c r="D254" s="2" t="n"/>
+      <c r="E254" s="2" t="n"/>
+      <c r="F254" s="2" t="n"/>
+      <c r="G254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n"/>
       <c r="B255" s="2" t="n"/>
       <c r="C255" s="2" t="n"/>
       <c r="D255" s="2" t="n"/>
+      <c r="E255" s="2" t="n"/>
+      <c r="F255" s="2" t="n"/>
+      <c r="G255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n"/>
       <c r="B256" s="2" t="n"/>
       <c r="C256" s="2" t="n"/>
       <c r="D256" s="2" t="n"/>
+      <c r="E256" s="2" t="n"/>
+      <c r="F256" s="2" t="n"/>
+      <c r="G256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n"/>
       <c r="B257" s="2" t="n"/>
       <c r="C257" s="2" t="n"/>
       <c r="D257" s="2" t="n"/>
+      <c r="E257" s="2" t="n"/>
+      <c r="F257" s="2" t="n"/>
+      <c r="G257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n"/>
       <c r="B258" s="2" t="n"/>
       <c r="C258" s="2" t="n"/>
       <c r="D258" s="2" t="n"/>
+      <c r="E258" s="2" t="n"/>
+      <c r="F258" s="2" t="n"/>
+      <c r="G258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n"/>
       <c r="B259" s="2" t="n"/>
       <c r="C259" s="2" t="n"/>
       <c r="D259" s="2" t="n"/>
+      <c r="E259" s="2" t="n"/>
+      <c r="F259" s="2" t="n"/>
+      <c r="G259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n"/>
       <c r="B260" s="2" t="n"/>
       <c r="C260" s="2" t="n"/>
       <c r="D260" s="2" t="n"/>
+      <c r="E260" s="2" t="n"/>
+      <c r="F260" s="2" t="n"/>
+      <c r="G260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n"/>
       <c r="B261" s="2" t="n"/>
       <c r="C261" s="2" t="n"/>
       <c r="D261" s="2" t="n"/>
+      <c r="E261" s="2" t="n"/>
+      <c r="F261" s="2" t="n"/>
+      <c r="G261" s="2" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n"/>
       <c r="B262" s="2" t="n"/>
       <c r="C262" s="2" t="n"/>
       <c r="D262" s="2" t="n"/>
+      <c r="E262" s="2" t="n"/>
+      <c r="F262" s="2" t="n"/>
+      <c r="G262" s="2" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n"/>
       <c r="B263" s="2" t="n"/>
       <c r="C263" s="2" t="n"/>
       <c r="D263" s="2" t="n"/>
+      <c r="E263" s="2" t="n"/>
+      <c r="F263" s="2" t="n"/>
+      <c r="G263" s="2" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n"/>
       <c r="B264" s="2" t="n"/>
       <c r="C264" s="2" t="n"/>
       <c r="D264" s="2" t="n"/>
+      <c r="E264" s="2" t="n"/>
+      <c r="F264" s="2" t="n"/>
+      <c r="G264" s="2" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n"/>
       <c r="B265" s="2" t="n"/>
       <c r="C265" s="2" t="n"/>
       <c r="D265" s="2" t="n"/>
+      <c r="E265" s="2" t="n"/>
+      <c r="F265" s="2" t="n"/>
+      <c r="G265" s="2" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n"/>
       <c r="B266" s="2" t="n"/>
       <c r="C266" s="2" t="n"/>
       <c r="D266" s="2" t="n"/>
+      <c r="E266" s="2" t="n"/>
+      <c r="F266" s="2" t="n"/>
+      <c r="G266" s="2" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n"/>
       <c r="B267" s="2" t="n"/>
       <c r="C267" s="2" t="n"/>
       <c r="D267" s="2" t="n"/>
+      <c r="E267" s="2" t="n"/>
+      <c r="F267" s="2" t="n"/>
+      <c r="G267" s="2" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n"/>
       <c r="B268" s="2" t="n"/>
       <c r="C268" s="2" t="n"/>
       <c r="D268" s="2" t="n"/>
+      <c r="E268" s="2" t="n"/>
+      <c r="F268" s="2" t="n"/>
+      <c r="G268" s="2" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n"/>
       <c r="B269" s="2" t="n"/>
       <c r="C269" s="2" t="n"/>
       <c r="D269" s="2" t="n"/>
+      <c r="E269" s="2" t="n"/>
+      <c r="F269" s="2" t="n"/>
+      <c r="G269" s="2" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n"/>
       <c r="B270" s="2" t="n"/>
       <c r="C270" s="2" t="n"/>
       <c r="D270" s="2" t="n"/>
+      <c r="E270" s="2" t="n"/>
+      <c r="F270" s="2" t="n"/>
+      <c r="G270" s="2" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n"/>
       <c r="B271" s="2" t="n"/>
       <c r="C271" s="2" t="n"/>
       <c r="D271" s="2" t="n"/>
+      <c r="E271" s="2" t="n"/>
+      <c r="F271" s="2" t="n"/>
+      <c r="G271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n"/>
       <c r="B272" s="2" t="n"/>
       <c r="C272" s="2" t="n"/>
       <c r="D272" s="2" t="n"/>
+      <c r="E272" s="2" t="n"/>
+      <c r="F272" s="2" t="n"/>
+      <c r="G272" s="2" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n"/>
       <c r="B273" s="2" t="n"/>
       <c r="C273" s="2" t="n"/>
       <c r="D273" s="2" t="n"/>
+      <c r="E273" s="2" t="n"/>
+      <c r="F273" s="2" t="n"/>
+      <c r="G273" s="2" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n"/>
       <c r="B274" s="2" t="n"/>
       <c r="C274" s="2" t="n"/>
       <c r="D274" s="2" t="n"/>
+      <c r="E274" s="2" t="n"/>
+      <c r="F274" s="2" t="n"/>
+      <c r="G274" s="2" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n"/>
       <c r="B275" s="2" t="n"/>
       <c r="C275" s="2" t="n"/>
       <c r="D275" s="2" t="n"/>
+      <c r="E275" s="2" t="n"/>
+      <c r="F275" s="2" t="n"/>
+      <c r="G275" s="2" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n"/>
       <c r="B276" s="2" t="n"/>
       <c r="C276" s="2" t="n"/>
       <c r="D276" s="2" t="n"/>
+      <c r="E276" s="2" t="n"/>
+      <c r="F276" s="2" t="n"/>
+      <c r="G276" s="2" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n"/>
       <c r="B277" s="2" t="n"/>
       <c r="C277" s="2" t="n"/>
       <c r="D277" s="2" t="n"/>
+      <c r="E277" s="2" t="n"/>
+      <c r="F277" s="2" t="n"/>
+      <c r="G277" s="2" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n"/>
       <c r="B278" s="2" t="n"/>
       <c r="C278" s="2" t="n"/>
       <c r="D278" s="2" t="n"/>
+      <c r="E278" s="2" t="n"/>
+      <c r="F278" s="2" t="n"/>
+      <c r="G278" s="2" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n"/>
       <c r="B279" s="2" t="n"/>
       <c r="C279" s="2" t="n"/>
       <c r="D279" s="2" t="n"/>
+      <c r="E279" s="2" t="n"/>
+      <c r="F279" s="2" t="n"/>
+      <c r="G279" s="2" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n"/>
       <c r="B280" s="2" t="n"/>
       <c r="C280" s="2" t="n"/>
       <c r="D280" s="2" t="n"/>
+      <c r="E280" s="2" t="n"/>
+      <c r="F280" s="2" t="n"/>
+      <c r="G280" s="2" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n"/>
       <c r="B281" s="2" t="n"/>
       <c r="C281" s="2" t="n"/>
       <c r="D281" s="2" t="n"/>
+      <c r="E281" s="2" t="n"/>
+      <c r="F281" s="2" t="n"/>
+      <c r="G281" s="2" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n"/>
       <c r="B282" s="2" t="n"/>
       <c r="C282" s="2" t="n"/>
       <c r="D282" s="2" t="n"/>
+      <c r="E282" s="2" t="n"/>
+      <c r="F282" s="2" t="n"/>
+      <c r="G282" s="2" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n"/>
       <c r="B283" s="2" t="n"/>
       <c r="C283" s="2" t="n"/>
       <c r="D283" s="2" t="n"/>
+      <c r="E283" s="2" t="n"/>
+      <c r="F283" s="2" t="n"/>
+      <c r="G283" s="2" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n"/>
       <c r="B284" s="2" t="n"/>
       <c r="C284" s="2" t="n"/>
       <c r="D284" s="2" t="n"/>
+      <c r="E284" s="2" t="n"/>
+      <c r="F284" s="2" t="n"/>
+      <c r="G284" s="2" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n"/>
       <c r="B285" s="2" t="n"/>
       <c r="C285" s="2" t="n"/>
       <c r="D285" s="2" t="n"/>
+      <c r="E285" s="2" t="n"/>
+      <c r="F285" s="2" t="n"/>
+      <c r="G285" s="2" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n"/>
       <c r="B286" s="2" t="n"/>
       <c r="C286" s="2" t="n"/>
       <c r="D286" s="2" t="n"/>
+      <c r="E286" s="2" t="n"/>
+      <c r="F286" s="2" t="n"/>
+      <c r="G286" s="2" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n"/>
       <c r="B287" s="2" t="n"/>
       <c r="C287" s="2" t="n"/>
       <c r="D287" s="2" t="n"/>
+      <c r="E287" s="2" t="n"/>
+      <c r="F287" s="2" t="n"/>
+      <c r="G287" s="2" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n"/>
       <c r="B288" s="2" t="n"/>
       <c r="C288" s="2" t="n"/>
       <c r="D288" s="2" t="n"/>
+      <c r="E288" s="2" t="n"/>
+      <c r="F288" s="2" t="n"/>
+      <c r="G288" s="2" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n"/>
       <c r="B289" s="2" t="n"/>
       <c r="C289" s="2" t="n"/>
       <c r="D289" s="2" t="n"/>
+      <c r="E289" s="2" t="n"/>
+      <c r="F289" s="2" t="n"/>
+      <c r="G289" s="2" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n"/>
       <c r="B290" s="2" t="n"/>
       <c r="C290" s="2" t="n"/>
       <c r="D290" s="2" t="n"/>
+      <c r="E290" s="2" t="n"/>
+      <c r="F290" s="2" t="n"/>
+      <c r="G290" s="2" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n"/>
       <c r="B291" s="2" t="n"/>
       <c r="C291" s="2" t="n"/>
       <c r="D291" s="2" t="n"/>
+      <c r="E291" s="2" t="n"/>
+      <c r="F291" s="2" t="n"/>
+      <c r="G291" s="2" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n"/>
       <c r="B292" s="2" t="n"/>
       <c r="C292" s="2" t="n"/>
       <c r="D292" s="2" t="n"/>
+      <c r="E292" s="2" t="n"/>
+      <c r="F292" s="2" t="n"/>
+      <c r="G292" s="2" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n"/>
       <c r="B293" s="2" t="n"/>
       <c r="C293" s="2" t="n"/>
       <c r="D293" s="2" t="n"/>
+      <c r="E293" s="2" t="n"/>
+      <c r="F293" s="2" t="n"/>
+      <c r="G293" s="2" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n"/>
       <c r="B294" s="2" t="n"/>
       <c r="C294" s="2" t="n"/>
       <c r="D294" s="2" t="n"/>
+      <c r="E294" s="2" t="n"/>
+      <c r="F294" s="2" t="n"/>
+      <c r="G294" s="2" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n"/>
       <c r="B295" s="2" t="n"/>
       <c r="C295" s="2" t="n"/>
       <c r="D295" s="2" t="n"/>
+      <c r="E295" s="2" t="n"/>
+      <c r="F295" s="2" t="n"/>
+      <c r="G295" s="2" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n"/>
       <c r="B296" s="2" t="n"/>
       <c r="C296" s="2" t="n"/>
       <c r="D296" s="2" t="n"/>
+      <c r="E296" s="2" t="n"/>
+      <c r="F296" s="2" t="n"/>
+      <c r="G296" s="2" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n"/>
       <c r="B297" s="2" t="n"/>
       <c r="C297" s="2" t="n"/>
       <c r="D297" s="2" t="n"/>
+      <c r="E297" s="2" t="n"/>
+      <c r="F297" s="2" t="n"/>
+      <c r="G297" s="2" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n"/>
       <c r="B298" s="2" t="n"/>
       <c r="C298" s="2" t="n"/>
       <c r="D298" s="2" t="n"/>
+      <c r="E298" s="2" t="n"/>
+      <c r="F298" s="2" t="n"/>
+      <c r="G298" s="2" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n"/>
       <c r="B299" s="2" t="n"/>
       <c r="C299" s="2" t="n"/>
       <c r="D299" s="2" t="n"/>
+      <c r="E299" s="2" t="n"/>
+      <c r="F299" s="2" t="n"/>
+      <c r="G299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n"/>
       <c r="B300" s="2" t="n"/>
       <c r="C300" s="2" t="n"/>
       <c r="D300" s="2" t="n"/>
+      <c r="E300" s="2" t="n"/>
+      <c r="F300" s="2" t="n"/>
+      <c r="G300" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="C2:D300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt datum" error="Skriv ett datum som ÅÅÅÅ-MM-DD, t.ex. 2026-11-03." prompt="Datum, t.ex. 2026-11-03. Lämna tomt för ingen gräns." type="date" operator="between">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
+    </dataValidation>
+    <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt värde" error="Välj ett värde i listan." prompt="Anslag (röd banderoll) eller Nyhet. Tomt = Anslag." type="list">
+      <formula1>"Anslag,Nyhet"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(#29): Klubbinfo tab in the sheet template
Headers, one row per setting with a Fält dropdown (reject invalid input),
Ort and the Facebook group prefilled. Other sheets are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Tränare" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Säsonger" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Anslag" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Klubbinfo" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14083,4 +14084,334 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fält</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Värde</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Värde (EN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Lokal</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Gatuadress</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Ronneby</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>E-post</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Telefon</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Bli medlem</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/251477413001</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Behold</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop">
+      <formula1>"Lokal,Gatuadress,Ort,E-post,Telefon,Bli medlem,Facebook,Instagram,Behold"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: several prices per group and several groups per session
- Grupper: rows with the same group name are one group with several
  prices (e.g. per term and per year). Details come from the first row
  that has them; identical and redundant free prices are dropped.
- Prices like "1 100,00 kr" are read as 1100, not 110000.
- Schema: Grupp may list several groups, comma-separated, like the
  Grupper column in Tränare. The filter, groups page, session card and
  start page handle it.
- Sheet template: Grupp in Schema is plain text, so comma lists aren't
  rejected. HOWTO explains both features.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -3733,15 +3733,12 @@
       <c r="H300" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt värde" error="Välj ett värde i listan." prompt="Välj veckodag" type="list">
       <formula1>"Måndag,Tisdag,Onsdag,Torsdag,Fredag,Lördag,Söndag"</formula1>
     </dataValidation>
     <dataValidation sqref="A2:A300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt värde" error="Välj ett värde i listan." prompt="Säsong från fliken Säsonger" type="list">
       <formula1>='Säsonger'!$A$2:$A$50</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt värde" error="Välj ett värde i listan." prompt="Grupp från fliken Grupper" type="list">
-      <formula1>='Grupper'!$A$2:$A$50</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ogiltigt värde" error="Välj ett värde i listan." prompt="Tränare från fliken Tränare" type="list">
       <formula1>='Tränare'!$A$2:$A$50</formula1>

</xml_diff>

<commit_message>
feat(#30): T4 Prova på tab in the sheet template and backup
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Säsonger" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Anslag" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Klubbinfo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prova på" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,12 +61,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -14411,4 +14415,1938 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D300"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Rubrik (EN)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Text (EN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Vad ska jag ha med mig?</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>What should I bring?</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Bekväma kläder och en vattenflaska räcker.
+- Träningskläder
+- Vattenflaska
+- Handduk
+Har du inga handskar? Fråga en tränare om att låna ett par.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Comfortable clothes and a water bottle are enough.
+- Training clothes
+- Water bottle
+- Towel
+No gloves? Ask a coach about borrowing a pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Första gången</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Your first time</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Kom ungefär 15 minuter innan passet börjar, så hinner vi visa dig runt.
+Passet börjar med uppvärmning och vi går igenom grunderna i lugn takt. Du bestämmer själv hur hårt du vill köra.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Arrive about 15 minutes before the session so we have time to show you around.
+Every session starts with a warm-up, and we go through the basics at a calm pace. You decide how hard you want to train.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Du behöver inte vara i form</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>You don't need to be fit</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Alla börjar någonstans. Träningen anpassas efter dig, och du kan ta pauser när du behöver.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Everyone starts somewhere. Training is adapted to you, and you can take breaks whenever you need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Föräldrar och vänner</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Det går bra att komma med och titta på ett pass. Fråga gärna en tränare på plats om du undrar något.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Vad kostar det?</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>What does it cost?</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Att prova på är gratis. Vill du fortsätta hittar du medlemskap och priser på gruppsidan: https://ronnebybk.github.io/ronneby-bk/#/grupper</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Trying a session is free. If you want to continue, membership and prices are on the groups page: https://ronnebybk.github.io/ronneby-bk/#/grupper</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Hur tar jag mig dit?</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>How do I get there?</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Lokalen och adressen hittar du på kontaktsidan: https://ronnebybk.github.io/ronneby-bk/#/kontakt</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>The venue and address are on the contact page: https://ronnebybk.github.io/ronneby-bk/#/kontakt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="2" t="n"/>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="2" t="n"/>
+      <c r="C98" s="2" t="n"/>
+      <c r="D98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="2" t="n"/>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n"/>
+      <c r="B100" s="2" t="n"/>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n"/>
+      <c r="B101" s="2" t="n"/>
+      <c r="C101" s="2" t="n"/>
+      <c r="D101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n"/>
+      <c r="B102" s="2" t="n"/>
+      <c r="C102" s="2" t="n"/>
+      <c r="D102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n"/>
+      <c r="B103" s="2" t="n"/>
+      <c r="C103" s="2" t="n"/>
+      <c r="D103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n"/>
+      <c r="B104" s="2" t="n"/>
+      <c r="C104" s="2" t="n"/>
+      <c r="D104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n"/>
+      <c r="B105" s="2" t="n"/>
+      <c r="C105" s="2" t="n"/>
+      <c r="D105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="2" t="n"/>
+      <c r="C106" s="2" t="n"/>
+      <c r="D106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n"/>
+      <c r="B107" s="2" t="n"/>
+      <c r="C107" s="2" t="n"/>
+      <c r="D107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="2" t="n"/>
+      <c r="C108" s="2" t="n"/>
+      <c r="D108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n"/>
+      <c r="B109" s="2" t="n"/>
+      <c r="C109" s="2" t="n"/>
+      <c r="D109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n"/>
+      <c r="B110" s="2" t="n"/>
+      <c r="C110" s="2" t="n"/>
+      <c r="D110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n"/>
+      <c r="B111" s="2" t="n"/>
+      <c r="C111" s="2" t="n"/>
+      <c r="D111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n"/>
+      <c r="B112" s="2" t="n"/>
+      <c r="C112" s="2" t="n"/>
+      <c r="D112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n"/>
+      <c r="B113" s="2" t="n"/>
+      <c r="C113" s="2" t="n"/>
+      <c r="D113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n"/>
+      <c r="B114" s="2" t="n"/>
+      <c r="C114" s="2" t="n"/>
+      <c r="D114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n"/>
+      <c r="B115" s="2" t="n"/>
+      <c r="C115" s="2" t="n"/>
+      <c r="D115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n"/>
+      <c r="B116" s="2" t="n"/>
+      <c r="C116" s="2" t="n"/>
+      <c r="D116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n"/>
+      <c r="B117" s="2" t="n"/>
+      <c r="C117" s="2" t="n"/>
+      <c r="D117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n"/>
+      <c r="B118" s="2" t="n"/>
+      <c r="C118" s="2" t="n"/>
+      <c r="D118" s="2" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n"/>
+      <c r="B119" s="2" t="n"/>
+      <c r="C119" s="2" t="n"/>
+      <c r="D119" s="2" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n"/>
+      <c r="B120" s="2" t="n"/>
+      <c r="C120" s="2" t="n"/>
+      <c r="D120" s="2" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n"/>
+      <c r="B121" s="2" t="n"/>
+      <c r="C121" s="2" t="n"/>
+      <c r="D121" s="2" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n"/>
+      <c r="B122" s="2" t="n"/>
+      <c r="C122" s="2" t="n"/>
+      <c r="D122" s="2" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n"/>
+      <c r="B123" s="2" t="n"/>
+      <c r="C123" s="2" t="n"/>
+      <c r="D123" s="2" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n"/>
+      <c r="B124" s="2" t="n"/>
+      <c r="C124" s="2" t="n"/>
+      <c r="D124" s="2" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n"/>
+      <c r="B125" s="2" t="n"/>
+      <c r="C125" s="2" t="n"/>
+      <c r="D125" s="2" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n"/>
+      <c r="B126" s="2" t="n"/>
+      <c r="C126" s="2" t="n"/>
+      <c r="D126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n"/>
+      <c r="B127" s="2" t="n"/>
+      <c r="C127" s="2" t="n"/>
+      <c r="D127" s="2" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n"/>
+      <c r="B128" s="2" t="n"/>
+      <c r="C128" s="2" t="n"/>
+      <c r="D128" s="2" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n"/>
+      <c r="B129" s="2" t="n"/>
+      <c r="C129" s="2" t="n"/>
+      <c r="D129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n"/>
+      <c r="B130" s="2" t="n"/>
+      <c r="C130" s="2" t="n"/>
+      <c r="D130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n"/>
+      <c r="B131" s="2" t="n"/>
+      <c r="C131" s="2" t="n"/>
+      <c r="D131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n"/>
+      <c r="B132" s="2" t="n"/>
+      <c r="C132" s="2" t="n"/>
+      <c r="D132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n"/>
+      <c r="B133" s="2" t="n"/>
+      <c r="C133" s="2" t="n"/>
+      <c r="D133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n"/>
+      <c r="B134" s="2" t="n"/>
+      <c r="C134" s="2" t="n"/>
+      <c r="D134" s="2" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n"/>
+      <c r="B135" s="2" t="n"/>
+      <c r="C135" s="2" t="n"/>
+      <c r="D135" s="2" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n"/>
+      <c r="B136" s="2" t="n"/>
+      <c r="C136" s="2" t="n"/>
+      <c r="D136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n"/>
+      <c r="B137" s="2" t="n"/>
+      <c r="C137" s="2" t="n"/>
+      <c r="D137" s="2" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n"/>
+      <c r="B138" s="2" t="n"/>
+      <c r="C138" s="2" t="n"/>
+      <c r="D138" s="2" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n"/>
+      <c r="B139" s="2" t="n"/>
+      <c r="C139" s="2" t="n"/>
+      <c r="D139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n"/>
+      <c r="B140" s="2" t="n"/>
+      <c r="C140" s="2" t="n"/>
+      <c r="D140" s="2" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n"/>
+      <c r="B141" s="2" t="n"/>
+      <c r="C141" s="2" t="n"/>
+      <c r="D141" s="2" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n"/>
+      <c r="B142" s="2" t="n"/>
+      <c r="C142" s="2" t="n"/>
+      <c r="D142" s="2" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n"/>
+      <c r="B143" s="2" t="n"/>
+      <c r="C143" s="2" t="n"/>
+      <c r="D143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n"/>
+      <c r="B144" s="2" t="n"/>
+      <c r="C144" s="2" t="n"/>
+      <c r="D144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n"/>
+      <c r="B145" s="2" t="n"/>
+      <c r="C145" s="2" t="n"/>
+      <c r="D145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n"/>
+      <c r="B146" s="2" t="n"/>
+      <c r="C146" s="2" t="n"/>
+      <c r="D146" s="2" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n"/>
+      <c r="B147" s="2" t="n"/>
+      <c r="C147" s="2" t="n"/>
+      <c r="D147" s="2" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n"/>
+      <c r="B148" s="2" t="n"/>
+      <c r="C148" s="2" t="n"/>
+      <c r="D148" s="2" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n"/>
+      <c r="B149" s="2" t="n"/>
+      <c r="C149" s="2" t="n"/>
+      <c r="D149" s="2" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n"/>
+      <c r="B150" s="2" t="n"/>
+      <c r="C150" s="2" t="n"/>
+      <c r="D150" s="2" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n"/>
+      <c r="B151" s="2" t="n"/>
+      <c r="C151" s="2" t="n"/>
+      <c r="D151" s="2" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n"/>
+      <c r="B152" s="2" t="n"/>
+      <c r="C152" s="2" t="n"/>
+      <c r="D152" s="2" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n"/>
+      <c r="B153" s="2" t="n"/>
+      <c r="C153" s="2" t="n"/>
+      <c r="D153" s="2" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n"/>
+      <c r="B154" s="2" t="n"/>
+      <c r="C154" s="2" t="n"/>
+      <c r="D154" s="2" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n"/>
+      <c r="B155" s="2" t="n"/>
+      <c r="C155" s="2" t="n"/>
+      <c r="D155" s="2" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n"/>
+      <c r="B156" s="2" t="n"/>
+      <c r="C156" s="2" t="n"/>
+      <c r="D156" s="2" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n"/>
+      <c r="B157" s="2" t="n"/>
+      <c r="C157" s="2" t="n"/>
+      <c r="D157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n"/>
+      <c r="B158" s="2" t="n"/>
+      <c r="C158" s="2" t="n"/>
+      <c r="D158" s="2" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n"/>
+      <c r="B159" s="2" t="n"/>
+      <c r="C159" s="2" t="n"/>
+      <c r="D159" s="2" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n"/>
+      <c r="B160" s="2" t="n"/>
+      <c r="C160" s="2" t="n"/>
+      <c r="D160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n"/>
+      <c r="B161" s="2" t="n"/>
+      <c r="C161" s="2" t="n"/>
+      <c r="D161" s="2" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n"/>
+      <c r="B162" s="2" t="n"/>
+      <c r="C162" s="2" t="n"/>
+      <c r="D162" s="2" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n"/>
+      <c r="B163" s="2" t="n"/>
+      <c r="C163" s="2" t="n"/>
+      <c r="D163" s="2" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n"/>
+      <c r="B164" s="2" t="n"/>
+      <c r="C164" s="2" t="n"/>
+      <c r="D164" s="2" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n"/>
+      <c r="B165" s="2" t="n"/>
+      <c r="C165" s="2" t="n"/>
+      <c r="D165" s="2" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n"/>
+      <c r="B166" s="2" t="n"/>
+      <c r="C166" s="2" t="n"/>
+      <c r="D166" s="2" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n"/>
+      <c r="B167" s="2" t="n"/>
+      <c r="C167" s="2" t="n"/>
+      <c r="D167" s="2" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n"/>
+      <c r="B168" s="2" t="n"/>
+      <c r="C168" s="2" t="n"/>
+      <c r="D168" s="2" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n"/>
+      <c r="B169" s="2" t="n"/>
+      <c r="C169" s="2" t="n"/>
+      <c r="D169" s="2" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n"/>
+      <c r="B170" s="2" t="n"/>
+      <c r="C170" s="2" t="n"/>
+      <c r="D170" s="2" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n"/>
+      <c r="B171" s="2" t="n"/>
+      <c r="C171" s="2" t="n"/>
+      <c r="D171" s="2" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n"/>
+      <c r="B172" s="2" t="n"/>
+      <c r="C172" s="2" t="n"/>
+      <c r="D172" s="2" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n"/>
+      <c r="B173" s="2" t="n"/>
+      <c r="C173" s="2" t="n"/>
+      <c r="D173" s="2" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n"/>
+      <c r="B174" s="2" t="n"/>
+      <c r="C174" s="2" t="n"/>
+      <c r="D174" s="2" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n"/>
+      <c r="B175" s="2" t="n"/>
+      <c r="C175" s="2" t="n"/>
+      <c r="D175" s="2" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n"/>
+      <c r="B176" s="2" t="n"/>
+      <c r="C176" s="2" t="n"/>
+      <c r="D176" s="2" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n"/>
+      <c r="B177" s="2" t="n"/>
+      <c r="C177" s="2" t="n"/>
+      <c r="D177" s="2" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n"/>
+      <c r="B178" s="2" t="n"/>
+      <c r="C178" s="2" t="n"/>
+      <c r="D178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n"/>
+      <c r="B179" s="2" t="n"/>
+      <c r="C179" s="2" t="n"/>
+      <c r="D179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n"/>
+      <c r="B180" s="2" t="n"/>
+      <c r="C180" s="2" t="n"/>
+      <c r="D180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n"/>
+      <c r="B181" s="2" t="n"/>
+      <c r="C181" s="2" t="n"/>
+      <c r="D181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n"/>
+      <c r="B182" s="2" t="n"/>
+      <c r="C182" s="2" t="n"/>
+      <c r="D182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n"/>
+      <c r="B183" s="2" t="n"/>
+      <c r="C183" s="2" t="n"/>
+      <c r="D183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n"/>
+      <c r="B184" s="2" t="n"/>
+      <c r="C184" s="2" t="n"/>
+      <c r="D184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n"/>
+      <c r="B185" s="2" t="n"/>
+      <c r="C185" s="2" t="n"/>
+      <c r="D185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n"/>
+      <c r="B186" s="2" t="n"/>
+      <c r="C186" s="2" t="n"/>
+      <c r="D186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n"/>
+      <c r="B187" s="2" t="n"/>
+      <c r="C187" s="2" t="n"/>
+      <c r="D187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n"/>
+      <c r="B188" s="2" t="n"/>
+      <c r="C188" s="2" t="n"/>
+      <c r="D188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n"/>
+      <c r="B189" s="2" t="n"/>
+      <c r="C189" s="2" t="n"/>
+      <c r="D189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n"/>
+      <c r="B190" s="2" t="n"/>
+      <c r="C190" s="2" t="n"/>
+      <c r="D190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n"/>
+      <c r="B191" s="2" t="n"/>
+      <c r="C191" s="2" t="n"/>
+      <c r="D191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n"/>
+      <c r="B192" s="2" t="n"/>
+      <c r="C192" s="2" t="n"/>
+      <c r="D192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n"/>
+      <c r="B193" s="2" t="n"/>
+      <c r="C193" s="2" t="n"/>
+      <c r="D193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n"/>
+      <c r="B194" s="2" t="n"/>
+      <c r="C194" s="2" t="n"/>
+      <c r="D194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n"/>
+      <c r="B195" s="2" t="n"/>
+      <c r="C195" s="2" t="n"/>
+      <c r="D195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n"/>
+      <c r="B196" s="2" t="n"/>
+      <c r="C196" s="2" t="n"/>
+      <c r="D196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n"/>
+      <c r="B197" s="2" t="n"/>
+      <c r="C197" s="2" t="n"/>
+      <c r="D197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n"/>
+      <c r="B198" s="2" t="n"/>
+      <c r="C198" s="2" t="n"/>
+      <c r="D198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n"/>
+      <c r="B199" s="2" t="n"/>
+      <c r="C199" s="2" t="n"/>
+      <c r="D199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n"/>
+      <c r="B200" s="2" t="n"/>
+      <c r="C200" s="2" t="n"/>
+      <c r="D200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n"/>
+      <c r="B201" s="2" t="n"/>
+      <c r="C201" s="2" t="n"/>
+      <c r="D201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n"/>
+      <c r="B202" s="2" t="n"/>
+      <c r="C202" s="2" t="n"/>
+      <c r="D202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n"/>
+      <c r="B203" s="2" t="n"/>
+      <c r="C203" s="2" t="n"/>
+      <c r="D203" s="2" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n"/>
+      <c r="B204" s="2" t="n"/>
+      <c r="C204" s="2" t="n"/>
+      <c r="D204" s="2" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n"/>
+      <c r="B205" s="2" t="n"/>
+      <c r="C205" s="2" t="n"/>
+      <c r="D205" s="2" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n"/>
+      <c r="B206" s="2" t="n"/>
+      <c r="C206" s="2" t="n"/>
+      <c r="D206" s="2" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n"/>
+      <c r="B207" s="2" t="n"/>
+      <c r="C207" s="2" t="n"/>
+      <c r="D207" s="2" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n"/>
+      <c r="B208" s="2" t="n"/>
+      <c r="C208" s="2" t="n"/>
+      <c r="D208" s="2" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n"/>
+      <c r="B209" s="2" t="n"/>
+      <c r="C209" s="2" t="n"/>
+      <c r="D209" s="2" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n"/>
+      <c r="B210" s="2" t="n"/>
+      <c r="C210" s="2" t="n"/>
+      <c r="D210" s="2" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n"/>
+      <c r="B211" s="2" t="n"/>
+      <c r="C211" s="2" t="n"/>
+      <c r="D211" s="2" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n"/>
+      <c r="B212" s="2" t="n"/>
+      <c r="C212" s="2" t="n"/>
+      <c r="D212" s="2" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n"/>
+      <c r="B213" s="2" t="n"/>
+      <c r="C213" s="2" t="n"/>
+      <c r="D213" s="2" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n"/>
+      <c r="B214" s="2" t="n"/>
+      <c r="C214" s="2" t="n"/>
+      <c r="D214" s="2" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n"/>
+      <c r="B215" s="2" t="n"/>
+      <c r="C215" s="2" t="n"/>
+      <c r="D215" s="2" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n"/>
+      <c r="B216" s="2" t="n"/>
+      <c r="C216" s="2" t="n"/>
+      <c r="D216" s="2" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n"/>
+      <c r="B217" s="2" t="n"/>
+      <c r="C217" s="2" t="n"/>
+      <c r="D217" s="2" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n"/>
+      <c r="B218" s="2" t="n"/>
+      <c r="C218" s="2" t="n"/>
+      <c r="D218" s="2" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n"/>
+      <c r="B219" s="2" t="n"/>
+      <c r="C219" s="2" t="n"/>
+      <c r="D219" s="2" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n"/>
+      <c r="B220" s="2" t="n"/>
+      <c r="C220" s="2" t="n"/>
+      <c r="D220" s="2" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n"/>
+      <c r="B221" s="2" t="n"/>
+      <c r="C221" s="2" t="n"/>
+      <c r="D221" s="2" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n"/>
+      <c r="B222" s="2" t="n"/>
+      <c r="C222" s="2" t="n"/>
+      <c r="D222" s="2" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n"/>
+      <c r="B223" s="2" t="n"/>
+      <c r="C223" s="2" t="n"/>
+      <c r="D223" s="2" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n"/>
+      <c r="B224" s="2" t="n"/>
+      <c r="C224" s="2" t="n"/>
+      <c r="D224" s="2" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n"/>
+      <c r="B225" s="2" t="n"/>
+      <c r="C225" s="2" t="n"/>
+      <c r="D225" s="2" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n"/>
+      <c r="B226" s="2" t="n"/>
+      <c r="C226" s="2" t="n"/>
+      <c r="D226" s="2" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n"/>
+      <c r="B227" s="2" t="n"/>
+      <c r="C227" s="2" t="n"/>
+      <c r="D227" s="2" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n"/>
+      <c r="B228" s="2" t="n"/>
+      <c r="C228" s="2" t="n"/>
+      <c r="D228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n"/>
+      <c r="B229" s="2" t="n"/>
+      <c r="C229" s="2" t="n"/>
+      <c r="D229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n"/>
+      <c r="B230" s="2" t="n"/>
+      <c r="C230" s="2" t="n"/>
+      <c r="D230" s="2" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n"/>
+      <c r="B231" s="2" t="n"/>
+      <c r="C231" s="2" t="n"/>
+      <c r="D231" s="2" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n"/>
+      <c r="B232" s="2" t="n"/>
+      <c r="C232" s="2" t="n"/>
+      <c r="D232" s="2" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n"/>
+      <c r="B233" s="2" t="n"/>
+      <c r="C233" s="2" t="n"/>
+      <c r="D233" s="2" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n"/>
+      <c r="B234" s="2" t="n"/>
+      <c r="C234" s="2" t="n"/>
+      <c r="D234" s="2" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n"/>
+      <c r="B235" s="2" t="n"/>
+      <c r="C235" s="2" t="n"/>
+      <c r="D235" s="2" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n"/>
+      <c r="B236" s="2" t="n"/>
+      <c r="C236" s="2" t="n"/>
+      <c r="D236" s="2" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n"/>
+      <c r="B237" s="2" t="n"/>
+      <c r="C237" s="2" t="n"/>
+      <c r="D237" s="2" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n"/>
+      <c r="B238" s="2" t="n"/>
+      <c r="C238" s="2" t="n"/>
+      <c r="D238" s="2" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n"/>
+      <c r="B239" s="2" t="n"/>
+      <c r="C239" s="2" t="n"/>
+      <c r="D239" s="2" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n"/>
+      <c r="B240" s="2" t="n"/>
+      <c r="C240" s="2" t="n"/>
+      <c r="D240" s="2" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n"/>
+      <c r="B241" s="2" t="n"/>
+      <c r="C241" s="2" t="n"/>
+      <c r="D241" s="2" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n"/>
+      <c r="B242" s="2" t="n"/>
+      <c r="C242" s="2" t="n"/>
+      <c r="D242" s="2" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n"/>
+      <c r="B243" s="2" t="n"/>
+      <c r="C243" s="2" t="n"/>
+      <c r="D243" s="2" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n"/>
+      <c r="B244" s="2" t="n"/>
+      <c r="C244" s="2" t="n"/>
+      <c r="D244" s="2" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n"/>
+      <c r="B245" s="2" t="n"/>
+      <c r="C245" s="2" t="n"/>
+      <c r="D245" s="2" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n"/>
+      <c r="B246" s="2" t="n"/>
+      <c r="C246" s="2" t="n"/>
+      <c r="D246" s="2" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n"/>
+      <c r="B247" s="2" t="n"/>
+      <c r="C247" s="2" t="n"/>
+      <c r="D247" s="2" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n"/>
+      <c r="B248" s="2" t="n"/>
+      <c r="C248" s="2" t="n"/>
+      <c r="D248" s="2" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n"/>
+      <c r="B249" s="2" t="n"/>
+      <c r="C249" s="2" t="n"/>
+      <c r="D249" s="2" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n"/>
+      <c r="B250" s="2" t="n"/>
+      <c r="C250" s="2" t="n"/>
+      <c r="D250" s="2" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n"/>
+      <c r="B251" s="2" t="n"/>
+      <c r="C251" s="2" t="n"/>
+      <c r="D251" s="2" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n"/>
+      <c r="B252" s="2" t="n"/>
+      <c r="C252" s="2" t="n"/>
+      <c r="D252" s="2" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n"/>
+      <c r="B253" s="2" t="n"/>
+      <c r="C253" s="2" t="n"/>
+      <c r="D253" s="2" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n"/>
+      <c r="B254" s="2" t="n"/>
+      <c r="C254" s="2" t="n"/>
+      <c r="D254" s="2" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n"/>
+      <c r="B255" s="2" t="n"/>
+      <c r="C255" s="2" t="n"/>
+      <c r="D255" s="2" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n"/>
+      <c r="B256" s="2" t="n"/>
+      <c r="C256" s="2" t="n"/>
+      <c r="D256" s="2" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n"/>
+      <c r="B257" s="2" t="n"/>
+      <c r="C257" s="2" t="n"/>
+      <c r="D257" s="2" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n"/>
+      <c r="B258" s="2" t="n"/>
+      <c r="C258" s="2" t="n"/>
+      <c r="D258" s="2" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n"/>
+      <c r="B259" s="2" t="n"/>
+      <c r="C259" s="2" t="n"/>
+      <c r="D259" s="2" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n"/>
+      <c r="B260" s="2" t="n"/>
+      <c r="C260" s="2" t="n"/>
+      <c r="D260" s="2" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n"/>
+      <c r="B261" s="2" t="n"/>
+      <c r="C261" s="2" t="n"/>
+      <c r="D261" s="2" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n"/>
+      <c r="B262" s="2" t="n"/>
+      <c r="C262" s="2" t="n"/>
+      <c r="D262" s="2" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n"/>
+      <c r="B263" s="2" t="n"/>
+      <c r="C263" s="2" t="n"/>
+      <c r="D263" s="2" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n"/>
+      <c r="B264" s="2" t="n"/>
+      <c r="C264" s="2" t="n"/>
+      <c r="D264" s="2" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n"/>
+      <c r="B265" s="2" t="n"/>
+      <c r="C265" s="2" t="n"/>
+      <c r="D265" s="2" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="n"/>
+      <c r="B266" s="2" t="n"/>
+      <c r="C266" s="2" t="n"/>
+      <c r="D266" s="2" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n"/>
+      <c r="B267" s="2" t="n"/>
+      <c r="C267" s="2" t="n"/>
+      <c r="D267" s="2" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n"/>
+      <c r="B268" s="2" t="n"/>
+      <c r="C268" s="2" t="n"/>
+      <c r="D268" s="2" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n"/>
+      <c r="B269" s="2" t="n"/>
+      <c r="C269" s="2" t="n"/>
+      <c r="D269" s="2" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n"/>
+      <c r="B270" s="2" t="n"/>
+      <c r="C270" s="2" t="n"/>
+      <c r="D270" s="2" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n"/>
+      <c r="B271" s="2" t="n"/>
+      <c r="C271" s="2" t="n"/>
+      <c r="D271" s="2" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n"/>
+      <c r="B272" s="2" t="n"/>
+      <c r="C272" s="2" t="n"/>
+      <c r="D272" s="2" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n"/>
+      <c r="B273" s="2" t="n"/>
+      <c r="C273" s="2" t="n"/>
+      <c r="D273" s="2" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n"/>
+      <c r="B274" s="2" t="n"/>
+      <c r="C274" s="2" t="n"/>
+      <c r="D274" s="2" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n"/>
+      <c r="B275" s="2" t="n"/>
+      <c r="C275" s="2" t="n"/>
+      <c r="D275" s="2" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n"/>
+      <c r="B276" s="2" t="n"/>
+      <c r="C276" s="2" t="n"/>
+      <c r="D276" s="2" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n"/>
+      <c r="B277" s="2" t="n"/>
+      <c r="C277" s="2" t="n"/>
+      <c r="D277" s="2" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n"/>
+      <c r="B278" s="2" t="n"/>
+      <c r="C278" s="2" t="n"/>
+      <c r="D278" s="2" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n"/>
+      <c r="B279" s="2" t="n"/>
+      <c r="C279" s="2" t="n"/>
+      <c r="D279" s="2" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n"/>
+      <c r="B280" s="2" t="n"/>
+      <c r="C280" s="2" t="n"/>
+      <c r="D280" s="2" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="n"/>
+      <c r="B281" s="2" t="n"/>
+      <c r="C281" s="2" t="n"/>
+      <c r="D281" s="2" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n"/>
+      <c r="B282" s="2" t="n"/>
+      <c r="C282" s="2" t="n"/>
+      <c r="D282" s="2" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="n"/>
+      <c r="B283" s="2" t="n"/>
+      <c r="C283" s="2" t="n"/>
+      <c r="D283" s="2" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="n"/>
+      <c r="B284" s="2" t="n"/>
+      <c r="C284" s="2" t="n"/>
+      <c r="D284" s="2" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="n"/>
+      <c r="B285" s="2" t="n"/>
+      <c r="C285" s="2" t="n"/>
+      <c r="D285" s="2" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="n"/>
+      <c r="B286" s="2" t="n"/>
+      <c r="C286" s="2" t="n"/>
+      <c r="D286" s="2" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="n"/>
+      <c r="B287" s="2" t="n"/>
+      <c r="C287" s="2" t="n"/>
+      <c r="D287" s="2" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n"/>
+      <c r="B288" s="2" t="n"/>
+      <c r="C288" s="2" t="n"/>
+      <c r="D288" s="2" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="n"/>
+      <c r="B289" s="2" t="n"/>
+      <c r="C289" s="2" t="n"/>
+      <c r="D289" s="2" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n"/>
+      <c r="B290" s="2" t="n"/>
+      <c r="C290" s="2" t="n"/>
+      <c r="D290" s="2" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="n"/>
+      <c r="B291" s="2" t="n"/>
+      <c r="C291" s="2" t="n"/>
+      <c r="D291" s="2" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="n"/>
+      <c r="B292" s="2" t="n"/>
+      <c r="C292" s="2" t="n"/>
+      <c r="D292" s="2" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="n"/>
+      <c r="B293" s="2" t="n"/>
+      <c r="C293" s="2" t="n"/>
+      <c r="D293" s="2" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="n"/>
+      <c r="B294" s="2" t="n"/>
+      <c r="C294" s="2" t="n"/>
+      <c r="D294" s="2" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="n"/>
+      <c r="B295" s="2" t="n"/>
+      <c r="C295" s="2" t="n"/>
+      <c r="D295" s="2" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="n"/>
+      <c r="B296" s="2" t="n"/>
+      <c r="C296" s="2" t="n"/>
+      <c r="D296" s="2" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="n"/>
+      <c r="B297" s="2" t="n"/>
+      <c r="C297" s="2" t="n"/>
+      <c r="D297" s="2" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="n"/>
+      <c r="B298" s="2" t="n"/>
+      <c r="C298" s="2" t="n"/>
+      <c r="D298" s="2" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="n"/>
+      <c r="B299" s="2" t="n"/>
+      <c r="C299" s="2" t="n"/>
+      <c r="D299" s="2" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="n"/>
+      <c r="B300" s="2" t="n"/>
+      <c r="C300" s="2" t="n"/>
+      <c r="D300" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(#30): keep the Prova på example text in one wording
The built-in text in sv.js/en.js is now the source for the demo rows
and the template: "Första gången" said "15 minuter" in one place and
"några minuter" in another. Links use #/grupper and #/kontakt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -14497,14 +14497,14 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Kom ungefär 15 minuter innan passet börjar, så hinner vi visa dig runt.
-Passet börjar med uppvärmning och vi går igenom grunderna i lugn takt. Du bestämmer själv hur hårt du vill köra.</t>
+          <t>Kom gärna några minuter innan passet börjar och säg till en tränare att du är ny.
+Vi visar dig vad du behöver veta, och du kan ta det i din egen takt.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Arrive about 15 minutes before the session so we have time to show you around.
-Every session starts with a warm-up, and we go through the basics at a calm pace. You decide how hard you want to train.</t>
+          <t>Arrive a few minutes before the session and tell a coach that you are new.
+We will show you what you need to know, and you can take it at your own pace.</t>
         </is>
       </c>
     </row>
@@ -14521,12 +14521,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Alla börjar någonstans. Träningen anpassas efter dig, och du kan ta pauser när du behöver.</t>
+          <t>Alla börjar någonstans. Säg till om du behöver ta en paus.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Everyone starts somewhere. Training is adapted to you, and you can take breaks whenever you need.</t>
+          <t>Everyone starts somewhere. Tell us if you need to take a break.</t>
         </is>
       </c>
     </row>
@@ -14536,13 +14536,21 @@
           <t>Föräldrar och vänner</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Parents and friends</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Det går bra att komma med och titta på ett pass. Fråga gärna en tränare på plats om du undrar något.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n"/>
+          <t>Vill du följa med och titta? Fråga en tränare på plats.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Would you like to come and watch? Ask a coach on site.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -14557,12 +14565,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Att prova på är gratis. Vill du fortsätta hittar du medlemskap och priser på gruppsidan: https://ronnebybk.github.io/ronneby-bk/#/grupper</t>
+          <t>Att prova på är gratis. Medlemskap och priser hittar du på #/grupper.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Trying a session is free. If you want to continue, membership and prices are on the groups page: https://ronnebybk.github.io/ronneby-bk/#/grupper</t>
+          <t>Trying a session is free. Membership and prices are under #/grupper.</t>
         </is>
       </c>
     </row>
@@ -14579,12 +14587,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Lokalen och adressen hittar du på kontaktsidan: https://ronnebybk.github.io/ronneby-bk/#/kontakt</t>
+          <t>Lokalen och adressen hittar du under #/kontakt.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>The venue and address are on the contact page: https://ronnebybk.github.io/ronneby-bk/#/kontakt</t>
+          <t>The venue and address are under #/kontakt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(#34): T4 Dokument tab in admin, backup and sheet template
Generated by Mistral Vibe.
Co-Authored-By: Mistral Vibe <vibe@mistral.ai>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Anslag" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Klubbinfo" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Prova på" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Frågor" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Frågor" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dokument" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -71,6 +72,7 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -16432,7 +16434,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vi har grupper från 8 år och uppåt:
+          <t>Vi har grupper från 8 år och uppåt:
 - Knattar: 8–12 år
 - Nybörjare: från 13 år
 - Tävling: från 15 år</t>
@@ -16440,7 +16442,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">We have groups from age 8 and up:
+          <t>We have groups from age 8 and up:
 - Kids: 8–12
 - Beginners: from 13
 - Competition: from 15</t>
@@ -18248,4 +18250,112 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Kategori (EN)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Titel (EN)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Beskrivning</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Beskrivning (EN)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Länk</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Regler</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gymregler</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gym rules</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Gäller för alla som tränar i lokalen.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Applies to everyone training in the venue.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/EXEMPEL/view?usp=sharing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ogiltigt datum" error="Ange ett giltigt datum (t.ex. 2026-03-15)." type="date" operator="greaterThanOrEqual">
+      <formula1>DATE(2000,1,1)</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(#35): T3 Resultat tab in the sheet template, admin and backup
Generated by Mistral Vibe.
Co-Authored-By: Mistral Vibe <vibe@mistral.ai>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Anslag" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Klubbinfo" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Prova på" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Frågor" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Frågor" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Resultat" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16432,7 +16433,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vi har grupper från 8 år och uppåt:
+          <t>Vi har grupper från 8 år och uppåt:
 - Knattar: 8–12 år
 - Nybörjare: från 13 år
 - Tävling: från 15 år</t>
@@ -16440,7 +16441,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">We have groups from age 8 and up:
+          <t>We have groups from age 8 and up:
 - Kids: 8–12
 - Beginners: from 13
 - Competition: from 15</t>
@@ -18248,4 +18249,93 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tävling</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tävling (EN)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Namn</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Junior/Senior</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Klass</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Klass (EN)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Placering</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Placering (EN)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Länk</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ej tillåtet värde" error="Välj Junior eller Senior i listan." prompt="Junior = bara förnamnet visas på hemsidan. Senior = hela namnet kan visas." type="list" errorStyle="stop">
+      <formula1>"Junior,Senior"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changed xlsx file. added small translation
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -14210,12 +14210,20 @@
       <c r="C10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Affisch märke</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Affisch prova på</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
     </row>
@@ -14412,7 +14420,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop">
-      <formula1>"Lokal,Gatuadress,Ort,E-post,Telefon,Bli medlem,Facebook,Instagram,Behold"</formula1>
+      <formula1>"Lokal,Gatuadress,Ort,E-post,Telefon,Bli medlem,Facebook,Instagram,Behold,Affisch märke,Affisch prova på"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(#36): T5 Sponsorer tab in the template and HOWTO
Generated by Mistral Vibe.
Co-Authored-By: Mistral Vibe <vibe@mistral.ai>
</commit_message>
<xml_diff>
--- a/sheet-template/ronneby-boxing-team-mall.xlsx
+++ b/sheet-template/ronneby-boxing-team-mall.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Frågor" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Dokument" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Resultat" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Sponsorer" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3848,6 +3849,346 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E300"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Namn</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Logga</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Länk</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Beskrivning</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Beskrivning (EN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>